<commit_message>
Site guncellemesi - 09.10.2026 18:25
</commit_message>
<xml_diff>
--- a/app/borsa/geri-alim-programlari/data/geri-alim.xlsx
+++ b/app/borsa/geri-alim-programlari/data/geri-alim.xlsx
@@ -73,18 +73,18 @@
     <x:t>ULUUN</x:t>
   </x:si>
   <x:si>
+    <x:t>SOKE</x:t>
+  </x:si>
+  <x:si>
+    <x:t>QUICK</x:t>
+  </x:si>
+  <x:si>
+    <x:t>GENTS</x:t>
+  </x:si>
+  <x:si>
     <x:t>07.10.2026</x:t>
   </x:si>
   <x:si>
-    <x:t>SOKE</x:t>
-  </x:si>
-  <x:si>
-    <x:t>QUICK</x:t>
-  </x:si>
-  <x:si>
-    <x:t>GENTS</x:t>
-  </x:si>
-  <x:si>
     <x:t>SVGYO</x:t>
   </x:si>
   <x:si>
@@ -1112,6 +1112,9 @@
   </x:si>
   <x:si>
     <x:t>29.08.2024</x:t>
+  </x:si>
+  <x:si>
+    <x:t>09.10.2026</x:t>
   </x:si>
   <x:si>
     <x:t>PSGYO</x:t>
@@ -1619,7 +1622,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="I2" s="0">
-        <x:v>12.91</x:v>
+        <x:v>13.9</x:v>
       </x:c>
       <x:c r="J2" s="0">
         <x:v>0</x:v>
@@ -1651,7 +1654,7 @@
         <x:v>0.26</x:v>
       </x:c>
       <x:c r="I3" s="0">
-        <x:v>30.46</x:v>
+        <x:v>31</x:v>
       </x:c>
       <x:c r="J3" s="0">
         <x:v>32.34</x:v>
@@ -1686,7 +1689,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="I4" s="0">
-        <x:v>47.7</x:v>
+        <x:v>52.45</x:v>
       </x:c>
       <x:c r="J4" s="0">
         <x:v>0</x:v>
@@ -1700,7 +1703,7 @@
         <x:v>16</x:v>
       </x:c>
       <x:c r="C5" s="0">
-        <x:v>3400630</x:v>
+        <x:v>5648081</x:v>
       </x:c>
       <x:c r="D5" s="0">
         <x:v>75000000</x:v>
@@ -1709,33 +1712,33 @@
         <x:v>525000000</x:v>
       </x:c>
       <x:c r="F5" s="0">
-        <x:v>22727179</x:v>
+        <x:v>37908802</x:v>
       </x:c>
       <x:c r="G5" s="0">
         <x:v>10</x:v>
       </x:c>
       <x:c r="H5" s="0">
-        <x:v>0.45</x:v>
+        <x:v>0.75</x:v>
       </x:c>
       <x:c r="I5" s="0">
-        <x:v>6.98</x:v>
+        <x:v>6.9</x:v>
       </x:c>
       <x:c r="J5" s="0">
-        <x:v>6.68</x:v>
+        <x:v>6.71</x:v>
       </x:c>
       <x:c r="K5" s="0" t="s">
-        <x:v>19</x:v>
+        <x:v>12</x:v>
       </x:c>
     </x:row>
     <x:row r="6" spans="1:11">
       <x:c r="A6" s="0" t="s">
-        <x:v>20</x:v>
+        <x:v>19</x:v>
       </x:c>
       <x:c r="B6" s="0" t="s">
         <x:v>16</x:v>
       </x:c>
       <x:c r="C6" s="0">
-        <x:v>2425000</x:v>
+        <x:v>3120684</x:v>
       </x:c>
       <x:c r="D6" s="0">
         <x:v>30000000</x:v>
@@ -1744,27 +1747,27 @@
         <x:v>210000000</x:v>
       </x:c>
       <x:c r="F6" s="0">
-        <x:v>17158250</x:v>
+        <x:v>22296364</x:v>
       </x:c>
       <x:c r="G6" s="0">
         <x:v>7.76</x:v>
       </x:c>
       <x:c r="H6" s="0">
-        <x:v>0.63</x:v>
+        <x:v>0.81</x:v>
       </x:c>
       <x:c r="I6" s="0">
-        <x:v>7.99</x:v>
+        <x:v>7.92</x:v>
       </x:c>
       <x:c r="J6" s="0">
-        <x:v>7.08</x:v>
+        <x:v>7.14</x:v>
       </x:c>
       <x:c r="K6" s="0" t="s">
-        <x:v>19</x:v>
+        <x:v>12</x:v>
       </x:c>
     </x:row>
     <x:row r="7" spans="1:11">
       <x:c r="A7" s="0" t="s">
-        <x:v>21</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="B7" s="0" t="s">
         <x:v>16</x:v>
@@ -1788,7 +1791,7 @@
         <x:v>0.31</x:v>
       </x:c>
       <x:c r="I7" s="0">
-        <x:v>49.08</x:v>
+        <x:v>49.48</x:v>
       </x:c>
       <x:c r="J7" s="0">
         <x:v>47.54</x:v>
@@ -1799,7 +1802,7 @@
     </x:row>
     <x:row r="8" spans="1:11">
       <x:c r="A8" s="0" t="s">
-        <x:v>22</x:v>
+        <x:v>21</x:v>
       </x:c>
       <x:c r="B8" s="0" t="s">
         <x:v>16</x:v>
@@ -1823,13 +1826,13 @@
         <x:v>0.05</x:v>
       </x:c>
       <x:c r="I8" s="0">
-        <x:v>4.14</x:v>
+        <x:v>4.16</x:v>
       </x:c>
       <x:c r="J8" s="0">
         <x:v>4.21</x:v>
       </x:c>
       <x:c r="K8" s="0" t="s">
-        <x:v>19</x:v>
+        <x:v>22</x:v>
       </x:c>
     </x:row>
     <x:row r="9" spans="1:11">
@@ -1858,13 +1861,13 @@
         <x:v>0.3</x:v>
       </x:c>
       <x:c r="I9" s="0">
-        <x:v>3.34</x:v>
+        <x:v>3.2</x:v>
       </x:c>
       <x:c r="J9" s="0">
         <x:v>3.38</x:v>
       </x:c>
       <x:c r="K9" s="0" t="s">
-        <x:v>19</x:v>
+        <x:v>22</x:v>
       </x:c>
     </x:row>
     <x:row r="10" spans="1:11">
@@ -1893,7 +1896,7 @@
         <x:v>0.34</x:v>
       </x:c>
       <x:c r="I10" s="0">
-        <x:v>51.85</x:v>
+        <x:v>53.8</x:v>
       </x:c>
       <x:c r="J10" s="0">
         <x:v>52.68</x:v>
@@ -1928,13 +1931,13 @@
         <x:v>0.12</x:v>
       </x:c>
       <x:c r="I11" s="0">
-        <x:v>99.2</x:v>
+        <x:v>109.1</x:v>
       </x:c>
       <x:c r="J11" s="0">
         <x:v>85.19</x:v>
       </x:c>
       <x:c r="K11" s="0" t="s">
-        <x:v>19</x:v>
+        <x:v>22</x:v>
       </x:c>
     </x:row>
     <x:row r="12" spans="1:11">
@@ -1963,7 +1966,7 @@
         <x:v>0.03</x:v>
       </x:c>
       <x:c r="I12" s="0">
-        <x:v>21.72</x:v>
+        <x:v>21.2</x:v>
       </x:c>
       <x:c r="J12" s="0">
         <x:v>19.3</x:v>
@@ -1998,7 +2001,7 @@
         <x:v>4.2</x:v>
       </x:c>
       <x:c r="I13" s="0">
-        <x:v>7.25</x:v>
+        <x:v>7.37</x:v>
       </x:c>
       <x:c r="J13" s="0">
         <x:v>7.05</x:v>
@@ -2015,7 +2018,7 @@
         <x:v>27</x:v>
       </x:c>
       <x:c r="C14" s="0">
-        <x:v>425944</x:v>
+        <x:v>490875</x:v>
       </x:c>
       <x:c r="D14" s="0">
         <x:v>7000000</x:v>
@@ -2024,22 +2027,22 @@
         <x:v>150000000</x:v>
       </x:c>
       <x:c r="F14" s="0">
-        <x:v>7011108</x:v>
+        <x:v>8097404</x:v>
       </x:c>
       <x:c r="G14" s="0">
         <x:v>3.5</x:v>
       </x:c>
       <x:c r="H14" s="0">
-        <x:v>0.21</x:v>
+        <x:v>0.25</x:v>
       </x:c>
       <x:c r="I14" s="0">
-        <x:v>16.72</x:v>
+        <x:v>16.74</x:v>
       </x:c>
       <x:c r="J14" s="0">
-        <x:v>16.46</x:v>
+        <x:v>16.5</x:v>
       </x:c>
       <x:c r="K14" s="0" t="s">
-        <x:v>19</x:v>
+        <x:v>12</x:v>
       </x:c>
     </x:row>
     <x:row r="15" spans="1:11">
@@ -2068,13 +2071,13 @@
         <x:v>0.02</x:v>
       </x:c>
       <x:c r="I15" s="0">
-        <x:v>8.88</x:v>
+        <x:v>8.79</x:v>
       </x:c>
       <x:c r="J15" s="0">
         <x:v>8.64</x:v>
       </x:c>
       <x:c r="K15" s="0" t="s">
-        <x:v>19</x:v>
+        <x:v>22</x:v>
       </x:c>
     </x:row>
     <x:row r="16" spans="1:11">
@@ -2085,7 +2088,7 @@
         <x:v>27</x:v>
       </x:c>
       <x:c r="C16" s="0">
-        <x:v>265485</x:v>
+        <x:v>350031</x:v>
       </x:c>
       <x:c r="D16" s="0">
         <x:v>4000000</x:v>
@@ -2094,22 +2097,22 @@
         <x:v>100000000</x:v>
       </x:c>
       <x:c r="F16" s="0">
-        <x:v>7144755</x:v>
+        <x:v>9595743</x:v>
       </x:c>
       <x:c r="G16" s="0">
         <x:v>1.46</x:v>
       </x:c>
       <x:c r="H16" s="0">
-        <x:v>0.1</x:v>
+        <x:v>0.13</x:v>
       </x:c>
       <x:c r="I16" s="0">
-        <x:v>29.42</x:v>
+        <x:v>30.26</x:v>
       </x:c>
       <x:c r="J16" s="0">
-        <x:v>26.91</x:v>
+        <x:v>27.41</x:v>
       </x:c>
       <x:c r="K16" s="0" t="s">
-        <x:v>15</x:v>
+        <x:v>12</x:v>
       </x:c>
     </x:row>
     <x:row r="17" spans="1:11">
@@ -2138,7 +2141,7 @@
         <x:v>0.1</x:v>
       </x:c>
       <x:c r="I17" s="0">
-        <x:v>13.66</x:v>
+        <x:v>14.24</x:v>
       </x:c>
       <x:c r="J17" s="0">
         <x:v>10.38</x:v>
@@ -2155,7 +2158,7 @@
         <x:v>30</x:v>
       </x:c>
       <x:c r="C18" s="0">
-        <x:v>335996</x:v>
+        <x:v>355996</x:v>
       </x:c>
       <x:c r="D18" s="0">
         <x:v>15000000</x:v>
@@ -2164,22 +2167,22 @@
         <x:v>110000000</x:v>
       </x:c>
       <x:c r="F18" s="0">
-        <x:v>1789677</x:v>
+        <x:v>1899277</x:v>
       </x:c>
       <x:c r="G18" s="0">
         <x:v>3.74</x:v>
       </x:c>
       <x:c r="H18" s="0">
-        <x:v>0.08</x:v>
+        <x:v>0.09</x:v>
       </x:c>
       <x:c r="I18" s="0">
-        <x:v>5.5</x:v>
+        <x:v>5.51</x:v>
       </x:c>
       <x:c r="J18" s="0">
-        <x:v>5.33</x:v>
+        <x:v>5.34</x:v>
       </x:c>
       <x:c r="K18" s="0" t="s">
-        <x:v>19</x:v>
+        <x:v>12</x:v>
       </x:c>
     </x:row>
     <x:row r="19" spans="1:11">
@@ -2208,13 +2211,13 @@
         <x:v>0.03</x:v>
       </x:c>
       <x:c r="I19" s="0">
-        <x:v>3.29</x:v>
+        <x:v>3.35</x:v>
       </x:c>
       <x:c r="J19" s="0">
         <x:v>3.34</x:v>
       </x:c>
       <x:c r="K19" s="0" t="s">
-        <x:v>19</x:v>
+        <x:v>22</x:v>
       </x:c>
     </x:row>
     <x:row r="20" spans="1:11">
@@ -2243,7 +2246,7 @@
         <x:v>0.25</x:v>
       </x:c>
       <x:c r="I20" s="0">
-        <x:v>1.06</x:v>
+        <x:v>1.09</x:v>
       </x:c>
       <x:c r="J20" s="0">
         <x:v>1.03</x:v>
@@ -2278,7 +2281,7 @@
         <x:v>0.64</x:v>
       </x:c>
       <x:c r="I21" s="0">
-        <x:v>11.46</x:v>
+        <x:v>11.75</x:v>
       </x:c>
       <x:c r="J21" s="0">
         <x:v>12.59</x:v>
@@ -2313,7 +2316,7 @@
         <x:v>1.88</x:v>
       </x:c>
       <x:c r="I22" s="0">
-        <x:v>8.33</x:v>
+        <x:v>8.24</x:v>
       </x:c>
       <x:c r="J22" s="0">
         <x:v>8.51</x:v>
@@ -2330,7 +2333,7 @@
         <x:v>30</x:v>
       </x:c>
       <x:c r="C23" s="0">
-        <x:v>215000</x:v>
+        <x:v>220000</x:v>
       </x:c>
       <x:c r="D23" s="0">
         <x:v>5000000</x:v>
@@ -2339,7 +2342,7 @@
         <x:v>400000000</x:v>
       </x:c>
       <x:c r="F23" s="0">
-        <x:v>14218390</x:v>
+        <x:v>14541640</x:v>
       </x:c>
       <x:c r="G23" s="0">
         <x:v>1.55</x:v>
@@ -2348,13 +2351,13 @@
         <x:v>0.07</x:v>
       </x:c>
       <x:c r="I23" s="0">
-        <x:v>64.65</x:v>
+        <x:v>67.1</x:v>
       </x:c>
       <x:c r="J23" s="0">
-        <x:v>66.13</x:v>
+        <x:v>66.1</x:v>
       </x:c>
       <x:c r="K23" s="0" t="s">
-        <x:v>19</x:v>
+        <x:v>12</x:v>
       </x:c>
     </x:row>
     <x:row r="24" spans="1:11">
@@ -2365,7 +2368,7 @@
         <x:v>30</x:v>
       </x:c>
       <x:c r="C24" s="0">
-        <x:v>1881188</x:v>
+        <x:v>2081188</x:v>
       </x:c>
       <x:c r="D24" s="0">
         <x:v>20000000</x:v>
@@ -2374,22 +2377,22 @@
         <x:v>250000000</x:v>
       </x:c>
       <x:c r="F24" s="0">
-        <x:v>9152511</x:v>
+        <x:v>10072011</x:v>
       </x:c>
       <x:c r="G24" s="0">
         <x:v>1.78</x:v>
       </x:c>
       <x:c r="H24" s="0">
-        <x:v>0.17</x:v>
+        <x:v>0.19</x:v>
       </x:c>
       <x:c r="I24" s="0">
-        <x:v>4.62</x:v>
+        <x:v>5.08</x:v>
       </x:c>
       <x:c r="J24" s="0">
-        <x:v>4.87</x:v>
+        <x:v>4.84</x:v>
       </x:c>
       <x:c r="K24" s="0" t="s">
-        <x:v>19</x:v>
+        <x:v>12</x:v>
       </x:c>
     </x:row>
     <x:row r="25" spans="1:11">
@@ -2400,7 +2403,7 @@
         <x:v>30</x:v>
       </x:c>
       <x:c r="C25" s="0">
-        <x:v>341000</x:v>
+        <x:v>706000</x:v>
       </x:c>
       <x:c r="D25" s="0">
         <x:v>28481914</x:v>
@@ -2409,22 +2412,22 @@
         <x:v>1000000000</x:v>
       </x:c>
       <x:c r="F25" s="0">
-        <x:v>2774376</x:v>
+        <x:v>5599476</x:v>
       </x:c>
       <x:c r="G25" s="0">
         <x:v>4.55</x:v>
       </x:c>
       <x:c r="H25" s="0">
-        <x:v>0.05</x:v>
+        <x:v>0.11</x:v>
       </x:c>
       <x:c r="I25" s="0">
-        <x:v>7.78</x:v>
+        <x:v>8.05</x:v>
       </x:c>
       <x:c r="J25" s="0">
-        <x:v>8.14</x:v>
+        <x:v>7.93</x:v>
       </x:c>
       <x:c r="K25" s="0" t="s">
-        <x:v>19</x:v>
+        <x:v>12</x:v>
       </x:c>
     </x:row>
     <x:row r="26" spans="1:11">
@@ -2453,7 +2456,7 @@
         <x:v>0.13</x:v>
       </x:c>
       <x:c r="I26" s="0">
-        <x:v>74.2</x:v>
+        <x:v>81.6</x:v>
       </x:c>
       <x:c r="J26" s="0">
         <x:v>72.97</x:v>
@@ -2488,7 +2491,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="I27" s="0">
-        <x:v>50.05</x:v>
+        <x:v>47.44</x:v>
       </x:c>
       <x:c r="J27" s="0">
         <x:v>0</x:v>
@@ -2520,13 +2523,13 @@
         <x:v>0.15</x:v>
       </x:c>
       <x:c r="I28" s="0">
-        <x:v>4.27</x:v>
+        <x:v>4.25</x:v>
       </x:c>
       <x:c r="J28" s="0">
         <x:v>4.32</x:v>
       </x:c>
       <x:c r="K28" s="0" t="s">
-        <x:v>19</x:v>
+        <x:v>22</x:v>
       </x:c>
     </x:row>
     <x:row r="29" spans="1:11">
@@ -2537,7 +2540,7 @@
         <x:v>46</x:v>
       </x:c>
       <x:c r="C29" s="0">
-        <x:v>5409436</x:v>
+        <x:v>5529436</x:v>
       </x:c>
       <x:c r="D29" s="0">
         <x:v>11848341</x:v>
@@ -2546,22 +2549,22 @@
         <x:v>250000000</x:v>
       </x:c>
       <x:c r="F29" s="0">
-        <x:v>49955603</x:v>
+        <x:v>50966603</x:v>
       </x:c>
       <x:c r="G29" s="0">
         <x:v>1.69</x:v>
       </x:c>
       <x:c r="H29" s="0">
-        <x:v>0.77</x:v>
+        <x:v>0.79</x:v>
       </x:c>
       <x:c r="I29" s="0">
-        <x:v>8.46</x:v>
+        <x:v>8.64</x:v>
       </x:c>
       <x:c r="J29" s="0">
-        <x:v>9.23</x:v>
+        <x:v>9.22</x:v>
       </x:c>
       <x:c r="K29" s="0" t="s">
-        <x:v>19</x:v>
+        <x:v>12</x:v>
       </x:c>
     </x:row>
     <x:row r="30" spans="1:11">
@@ -2590,7 +2593,7 @@
         <x:v>1.13</x:v>
       </x:c>
       <x:c r="I30" s="0">
-        <x:v>7.57</x:v>
+        <x:v>7.76</x:v>
       </x:c>
       <x:c r="J30" s="0">
         <x:v>7.82</x:v>
@@ -2625,7 +2628,7 @@
         <x:v>2.7</x:v>
       </x:c>
       <x:c r="I31" s="0">
-        <x:v>7.25</x:v>
+        <x:v>7.37</x:v>
       </x:c>
       <x:c r="J31" s="0">
         <x:v>6.81</x:v>
@@ -2660,7 +2663,7 @@
         <x:v>0.51</x:v>
       </x:c>
       <x:c r="I32" s="0">
-        <x:v>1.6</x:v>
+        <x:v>1.62</x:v>
       </x:c>
       <x:c r="J32" s="0">
         <x:v>1.59</x:v>
@@ -2677,7 +2680,7 @@
         <x:v>49</x:v>
       </x:c>
       <x:c r="C33" s="0">
-        <x:v>275229</x:v>
+        <x:v>305229</x:v>
       </x:c>
       <x:c r="D33" s="0">
         <x:v>2000000</x:v>
@@ -2686,22 +2689,22 @@
         <x:v>40000000</x:v>
       </x:c>
       <x:c r="F33" s="0">
-        <x:v>3112058</x:v>
+        <x:v>3452978</x:v>
       </x:c>
       <x:c r="G33" s="0">
         <x:v>2.38</x:v>
       </x:c>
       <x:c r="H33" s="0">
-        <x:v>0.33</x:v>
+        <x:v>0.36</x:v>
       </x:c>
       <x:c r="I33" s="0">
-        <x:v>11.36</x:v>
+        <x:v>11.89</x:v>
       </x:c>
       <x:c r="J33" s="0">
         <x:v>11.31</x:v>
       </x:c>
       <x:c r="K33" s="0" t="s">
-        <x:v>19</x:v>
+        <x:v>12</x:v>
       </x:c>
     </x:row>
     <x:row r="34" spans="1:11">
@@ -2712,7 +2715,7 @@
         <x:v>49</x:v>
       </x:c>
       <x:c r="C34" s="0">
-        <x:v>5318015</x:v>
+        <x:v>6194766</x:v>
       </x:c>
       <x:c r="D34" s="0">
         <x:v>15000000</x:v>
@@ -2721,22 +2724,22 @@
         <x:v>50000000</x:v>
       </x:c>
       <x:c r="F34" s="0">
-        <x:v>11357225</x:v>
+        <x:v>13192265</x:v>
       </x:c>
       <x:c r="G34" s="0">
         <x:v>0.69</x:v>
       </x:c>
       <x:c r="H34" s="0">
-        <x:v>0.25</x:v>
+        <x:v>0.29</x:v>
       </x:c>
       <x:c r="I34" s="0">
-        <x:v>2.18</x:v>
+        <x:v>2.21</x:v>
       </x:c>
       <x:c r="J34" s="0">
-        <x:v>2.14</x:v>
+        <x:v>2.13</x:v>
       </x:c>
       <x:c r="K34" s="0" t="s">
-        <x:v>19</x:v>
+        <x:v>12</x:v>
       </x:c>
     </x:row>
     <x:row r="35" spans="1:11">
@@ -2765,13 +2768,13 @@
         <x:v>0.17</x:v>
       </x:c>
       <x:c r="I35" s="0">
-        <x:v>29.98</x:v>
+        <x:v>30.2</x:v>
       </x:c>
       <x:c r="J35" s="0">
         <x:v>29.29</x:v>
       </x:c>
       <x:c r="K35" s="0" t="s">
-        <x:v>19</x:v>
+        <x:v>22</x:v>
       </x:c>
     </x:row>
     <x:row r="36" spans="1:11">
@@ -2800,7 +2803,7 @@
         <x:v>0.04</x:v>
       </x:c>
       <x:c r="I36" s="0">
-        <x:v>72.75</x:v>
+        <x:v>75</x:v>
       </x:c>
       <x:c r="J36" s="0">
         <x:v>74.13</x:v>
@@ -2835,7 +2838,7 @@
         <x:v>0.61</x:v>
       </x:c>
       <x:c r="I37" s="0">
-        <x:v>50.3</x:v>
+        <x:v>51.5</x:v>
       </x:c>
       <x:c r="J37" s="0">
         <x:v>57.9</x:v>
@@ -2870,7 +2873,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="I38" s="0">
-        <x:v>38.92</x:v>
+        <x:v>38.98</x:v>
       </x:c>
       <x:c r="J38" s="0">
         <x:v>0</x:v>
@@ -2902,7 +2905,7 @@
         <x:v>0.66</x:v>
       </x:c>
       <x:c r="I39" s="0">
-        <x:v>125.9</x:v>
+        <x:v>123</x:v>
       </x:c>
       <x:c r="J39" s="0">
         <x:v>115.6</x:v>
@@ -2937,13 +2940,13 @@
         <x:v>0.42</x:v>
       </x:c>
       <x:c r="I40" s="0">
-        <x:v>3.06</x:v>
+        <x:v>3.2</x:v>
       </x:c>
       <x:c r="J40" s="0">
         <x:v>3.12</x:v>
       </x:c>
       <x:c r="K40" s="0" t="s">
-        <x:v>19</x:v>
+        <x:v>22</x:v>
       </x:c>
     </x:row>
     <x:row r="41" spans="1:11">
@@ -2954,7 +2957,7 @@
         <x:v>59</x:v>
       </x:c>
       <x:c r="C41" s="0">
-        <x:v>1853000</x:v>
+        <x:v>2136000</x:v>
       </x:c>
       <x:c r="D41" s="0">
         <x:v>5000000</x:v>
@@ -2963,22 +2966,22 @@
         <x:v>1000000000</x:v>
       </x:c>
       <x:c r="F41" s="0">
-        <x:v>223145353</x:v>
+        <x:v>254855503</x:v>
       </x:c>
       <x:c r="G41" s="0">
         <x:v>4</x:v>
       </x:c>
       <x:c r="H41" s="0">
-        <x:v>1.48</x:v>
+        <x:v>1.71</x:v>
       </x:c>
       <x:c r="I41" s="0">
-        <x:v>121.5</x:v>
+        <x:v>122</x:v>
       </x:c>
       <x:c r="J41" s="0">
-        <x:v>120.42</x:v>
+        <x:v>119.31</x:v>
       </x:c>
       <x:c r="K41" s="0" t="s">
-        <x:v>19</x:v>
+        <x:v>12</x:v>
       </x:c>
     </x:row>
     <x:row r="42" spans="1:11">
@@ -3007,7 +3010,7 @@
         <x:v>0.34</x:v>
       </x:c>
       <x:c r="I42" s="0">
-        <x:v>36.94</x:v>
+        <x:v>36.6</x:v>
       </x:c>
       <x:c r="J42" s="0">
         <x:v>37.34</x:v>
@@ -3077,7 +3080,7 @@
         <x:v>2.7</x:v>
       </x:c>
       <x:c r="I44" s="0">
-        <x:v>7.25</x:v>
+        <x:v>7.37</x:v>
       </x:c>
       <x:c r="J44" s="0">
         <x:v>6.81</x:v>
@@ -3094,7 +3097,7 @@
         <x:v>63</x:v>
       </x:c>
       <x:c r="C45" s="0">
-        <x:v>23944766</x:v>
+        <x:v>24896406</x:v>
       </x:c>
       <x:c r="D45" s="0">
         <x:v>50000000</x:v>
@@ -3103,22 +3106,22 @@
         <x:v>200000000</x:v>
       </x:c>
       <x:c r="F45" s="0">
-        <x:v>136190413</x:v>
+        <x:v>141706118</x:v>
       </x:c>
       <x:c r="G45" s="0">
         <x:v>4.63</x:v>
       </x:c>
       <x:c r="H45" s="0">
-        <x:v>2.22</x:v>
+        <x:v>2.31</x:v>
       </x:c>
       <x:c r="I45" s="0">
-        <x:v>5.8</x:v>
+        <x:v>5.88</x:v>
       </x:c>
       <x:c r="J45" s="0">
         <x:v>5.69</x:v>
       </x:c>
       <x:c r="K45" s="0" t="s">
-        <x:v>19</x:v>
+        <x:v>12</x:v>
       </x:c>
     </x:row>
     <x:row r="46" spans="1:11">
@@ -3147,7 +3150,7 @@
         <x:v>0.17</x:v>
       </x:c>
       <x:c r="I46" s="0">
-        <x:v>9.58</x:v>
+        <x:v>9.77</x:v>
       </x:c>
       <x:c r="J46" s="0">
         <x:v>9.96</x:v>
@@ -3182,7 +3185,7 @@
         <x:v>0.36</x:v>
       </x:c>
       <x:c r="I47" s="0">
-        <x:v>18.73</x:v>
+        <x:v>19.7</x:v>
       </x:c>
       <x:c r="J47" s="0">
         <x:v>20.88</x:v>
@@ -3217,13 +3220,13 @@
         <x:v>0.3</x:v>
       </x:c>
       <x:c r="I48" s="0">
-        <x:v>14.01</x:v>
+        <x:v>13.93</x:v>
       </x:c>
       <x:c r="J48" s="0">
         <x:v>13.84</x:v>
       </x:c>
       <x:c r="K48" s="0" t="s">
-        <x:v>19</x:v>
+        <x:v>22</x:v>
       </x:c>
     </x:row>
     <x:row r="49" spans="1:11">
@@ -3252,7 +3255,7 @@
         <x:v>0.37</x:v>
       </x:c>
       <x:c r="I49" s="0">
-        <x:v>32.7</x:v>
+        <x:v>32.2</x:v>
       </x:c>
       <x:c r="J49" s="0">
         <x:v>34.56</x:v>
@@ -3287,7 +3290,7 @@
         <x:v>0.71</x:v>
       </x:c>
       <x:c r="I50" s="0">
-        <x:v>6.82</x:v>
+        <x:v>6.92</x:v>
       </x:c>
       <x:c r="J50" s="0">
         <x:v>7.25</x:v>
@@ -3322,7 +3325,7 @@
         <x:v>0.26</x:v>
       </x:c>
       <x:c r="I51" s="0">
-        <x:v>30.46</x:v>
+        <x:v>31</x:v>
       </x:c>
       <x:c r="J51" s="0">
         <x:v>32.34</x:v>
@@ -3357,7 +3360,7 @@
         <x:v>0.33</x:v>
       </x:c>
       <x:c r="I52" s="0">
-        <x:v>3.35</x:v>
+        <x:v>3.55</x:v>
       </x:c>
       <x:c r="J52" s="0">
         <x:v>3.51</x:v>
@@ -3392,13 +3395,13 @@
         <x:v>3.78</x:v>
       </x:c>
       <x:c r="I53" s="0">
-        <x:v>1.99</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="J53" s="0">
         <x:v>2.14</x:v>
       </x:c>
       <x:c r="K53" s="0" t="s">
-        <x:v>19</x:v>
+        <x:v>22</x:v>
       </x:c>
     </x:row>
     <x:row r="54" spans="1:11">
@@ -3433,7 +3436,7 @@
         <x:v>8.33</x:v>
       </x:c>
       <x:c r="K54" s="0" t="s">
-        <x:v>19</x:v>
+        <x:v>22</x:v>
       </x:c>
     </x:row>
     <x:row r="55" spans="1:11">
@@ -3444,7 +3447,7 @@
         <x:v>73</x:v>
       </x:c>
       <x:c r="C55" s="0">
-        <x:v>3689298</x:v>
+        <x:v>3839798</x:v>
       </x:c>
       <x:c r="D55" s="0">
         <x:v>12000000</x:v>
@@ -3453,22 +3456,22 @@
         <x:v>600000000</x:v>
       </x:c>
       <x:c r="F55" s="0">
-        <x:v>138512360</x:v>
+        <x:v>144083118</x:v>
       </x:c>
       <x:c r="G55" s="0">
         <x:v>2.16</x:v>
       </x:c>
       <x:c r="H55" s="0">
-        <x:v>0.66</x:v>
+        <x:v>0.69</x:v>
       </x:c>
       <x:c r="I55" s="0">
-        <x:v>37.26</x:v>
+        <x:v>38.04</x:v>
       </x:c>
       <x:c r="J55" s="0">
-        <x:v>37.54</x:v>
+        <x:v>37.52</x:v>
       </x:c>
       <x:c r="K55" s="0" t="s">
-        <x:v>19</x:v>
+        <x:v>12</x:v>
       </x:c>
     </x:row>
     <x:row r="56" spans="1:11">
@@ -3497,7 +3500,7 @@
         <x:v>0.18</x:v>
       </x:c>
       <x:c r="I56" s="0">
-        <x:v>3.84</x:v>
+        <x:v>3.69</x:v>
       </x:c>
       <x:c r="J56" s="0">
         <x:v>3.78</x:v>
@@ -3514,7 +3517,7 @@
         <x:v>73</x:v>
       </x:c>
       <x:c r="C57" s="0">
-        <x:v>165000</x:v>
+        <x:v>200000</x:v>
       </x:c>
       <x:c r="D57" s="0">
         <x:v>5000000</x:v>
@@ -3523,22 +3526,22 @@
         <x:v>250000000</x:v>
       </x:c>
       <x:c r="F57" s="0">
-        <x:v>7525285</x:v>
+        <x:v>9105535</x:v>
       </x:c>
       <x:c r="G57" s="0">
         <x:v>0.92</x:v>
       </x:c>
       <x:c r="H57" s="0">
-        <x:v>0.03</x:v>
+        <x:v>0.04</x:v>
       </x:c>
       <x:c r="I57" s="0">
-        <x:v>45.36</x:v>
+        <x:v>43</x:v>
       </x:c>
       <x:c r="J57" s="0">
-        <x:v>45.61</x:v>
+        <x:v>45.53</x:v>
       </x:c>
       <x:c r="K57" s="0" t="s">
-        <x:v>19</x:v>
+        <x:v>12</x:v>
       </x:c>
     </x:row>
     <x:row r="58" spans="1:11">
@@ -3567,7 +3570,7 @@
         <x:v>0.24</x:v>
       </x:c>
       <x:c r="I58" s="0">
-        <x:v>22.5</x:v>
+        <x:v>22.26</x:v>
       </x:c>
       <x:c r="J58" s="0">
         <x:v>24.37</x:v>
@@ -3602,7 +3605,7 @@
         <x:v>0.11</x:v>
       </x:c>
       <x:c r="I59" s="0">
-        <x:v>4.25</x:v>
+        <x:v>4.67</x:v>
       </x:c>
       <x:c r="J59" s="0">
         <x:v>6.94</x:v>
@@ -3637,7 +3640,7 @@
         <x:v>2.38</x:v>
       </x:c>
       <x:c r="I60" s="0">
-        <x:v>7.92</x:v>
+        <x:v>8.01</x:v>
       </x:c>
       <x:c r="J60" s="0">
         <x:v>8.87</x:v>
@@ -3672,7 +3675,7 @@
         <x:v>1.67</x:v>
       </x:c>
       <x:c r="I61" s="0">
-        <x:v>5</x:v>
+        <x:v>5.04</x:v>
       </x:c>
       <x:c r="J61" s="0">
         <x:v>5.95</x:v>
@@ -3707,7 +3710,7 @@
         <x:v>0.09</x:v>
       </x:c>
       <x:c r="I62" s="0">
-        <x:v>34.5</x:v>
+        <x:v>35.44</x:v>
       </x:c>
       <x:c r="J62" s="0">
         <x:v>37.41</x:v>
@@ -3742,13 +3745,13 @@
         <x:v>4.22</x:v>
       </x:c>
       <x:c r="I63" s="0">
-        <x:v>124.2</x:v>
+        <x:v>119</x:v>
       </x:c>
       <x:c r="J63" s="0">
         <x:v>86.07</x:v>
       </x:c>
       <x:c r="K63" s="0" t="s">
-        <x:v>19</x:v>
+        <x:v>22</x:v>
       </x:c>
     </x:row>
     <x:row r="64" spans="1:11">
@@ -3759,7 +3762,7 @@
         <x:v>82</x:v>
       </x:c>
       <x:c r="C64" s="0">
-        <x:v>8520576</x:v>
+        <x:v>9780787</x:v>
       </x:c>
       <x:c r="D64" s="0">
         <x:v>100000000</x:v>
@@ -3768,22 +3771,22 @@
         <x:v>700000000</x:v>
       </x:c>
       <x:c r="F64" s="0">
-        <x:v>42873561</x:v>
+        <x:v>49180917</x:v>
       </x:c>
       <x:c r="G64" s="0">
         <x:v>5</x:v>
       </x:c>
       <x:c r="H64" s="0">
-        <x:v>0.43</x:v>
+        <x:v>0.49</x:v>
       </x:c>
       <x:c r="I64" s="0">
-        <x:v>5.03</x:v>
+        <x:v>4.92</x:v>
       </x:c>
       <x:c r="J64" s="0">
         <x:v>5.03</x:v>
       </x:c>
       <x:c r="K64" s="0" t="s">
-        <x:v>19</x:v>
+        <x:v>12</x:v>
       </x:c>
     </x:row>
     <x:row r="65" spans="1:11">
@@ -3794,7 +3797,7 @@
         <x:v>88</x:v>
       </x:c>
       <x:c r="C65" s="0">
-        <x:v>24301435</x:v>
+        <x:v>27555966</x:v>
       </x:c>
       <x:c r="D65" s="0">
         <x:v>60000000</x:v>
@@ -3803,22 +3806,22 @@
         <x:v>200000000</x:v>
       </x:c>
       <x:c r="F65" s="0">
-        <x:v>59665231</x:v>
+        <x:v>67384313</x:v>
       </x:c>
       <x:c r="G65" s="0">
         <x:v>1.54</x:v>
       </x:c>
       <x:c r="H65" s="0">
-        <x:v>0.62</x:v>
+        <x:v>0.71</x:v>
       </x:c>
       <x:c r="I65" s="0">
-        <x:v>2.4</x:v>
+        <x:v>2.46</x:v>
       </x:c>
       <x:c r="J65" s="0">
-        <x:v>2.46</x:v>
+        <x:v>2.45</x:v>
       </x:c>
       <x:c r="K65" s="0" t="s">
-        <x:v>19</x:v>
+        <x:v>12</x:v>
       </x:c>
     </x:row>
     <x:row r="66" spans="1:11">
@@ -3864,7 +3867,7 @@
         <x:v>88</x:v>
       </x:c>
       <x:c r="C67" s="0">
-        <x:v>116174</x:v>
+        <x:v>121130</x:v>
       </x:c>
       <x:c r="D67" s="0">
         <x:v>9260000</x:v>
@@ -3873,7 +3876,7 @@
         <x:v>1200000000</x:v>
       </x:c>
       <x:c r="F67" s="0">
-        <x:v>11359357</x:v>
+        <x:v>11864869</x:v>
       </x:c>
       <x:c r="G67" s="0">
         <x:v>10</x:v>
@@ -3882,13 +3885,13 @@
         <x:v>0.13</x:v>
       </x:c>
       <x:c r="I67" s="0">
-        <x:v>102.1</x:v>
+        <x:v>101.6</x:v>
       </x:c>
       <x:c r="J67" s="0">
-        <x:v>97.78</x:v>
+        <x:v>97.95</x:v>
       </x:c>
       <x:c r="K67" s="0" t="s">
-        <x:v>19</x:v>
+        <x:v>12</x:v>
       </x:c>
     </x:row>
     <x:row r="68" spans="1:11">
@@ -3899,7 +3902,7 @@
         <x:v>88</x:v>
       </x:c>
       <x:c r="C68" s="0">
-        <x:v>856204</x:v>
+        <x:v>1276630</x:v>
       </x:c>
       <x:c r="D68" s="0">
         <x:v>2500000</x:v>
@@ -3908,22 +3911,22 @@
         <x:v>225000000</x:v>
       </x:c>
       <x:c r="F68" s="0">
-        <x:v>61745274</x:v>
+        <x:v>93067011</x:v>
       </x:c>
       <x:c r="G68" s="0">
         <x:v>0.74</x:v>
       </x:c>
       <x:c r="H68" s="0">
-        <x:v>0.25</x:v>
+        <x:v>0.38</x:v>
       </x:c>
       <x:c r="I68" s="0">
-        <x:v>72.6</x:v>
+        <x:v>73.5</x:v>
       </x:c>
       <x:c r="J68" s="0">
-        <x:v>72.12</x:v>
+        <x:v>72.9</x:v>
       </x:c>
       <x:c r="K68" s="0" t="s">
-        <x:v>19</x:v>
+        <x:v>12</x:v>
       </x:c>
     </x:row>
     <x:row r="69" spans="1:11">
@@ -3934,7 +3937,7 @@
         <x:v>88</x:v>
       </x:c>
       <x:c r="C69" s="0">
-        <x:v>6972564</x:v>
+        <x:v>7537299</x:v>
       </x:c>
       <x:c r="D69" s="0">
         <x:v>50000000</x:v>
@@ -3943,22 +3946,22 @@
         <x:v>2000000000</x:v>
       </x:c>
       <x:c r="F69" s="0">
-        <x:v>295390414</x:v>
+        <x:v>322502212</x:v>
       </x:c>
       <x:c r="G69" s="0">
         <x:v>1.92</x:v>
       </x:c>
       <x:c r="H69" s="0">
-        <x:v>0.27</x:v>
+        <x:v>0.29</x:v>
       </x:c>
       <x:c r="I69" s="0">
-        <x:v>48.02</x:v>
+        <x:v>48.38</x:v>
       </x:c>
       <x:c r="J69" s="0">
-        <x:v>42.36</x:v>
+        <x:v>42.79</x:v>
       </x:c>
       <x:c r="K69" s="0" t="s">
-        <x:v>15</x:v>
+        <x:v>12</x:v>
       </x:c>
     </x:row>
     <x:row r="70" spans="1:11">
@@ -3969,7 +3972,7 @@
         <x:v>88</x:v>
       </x:c>
       <x:c r="C70" s="0">
-        <x:v>46035847</x:v>
+        <x:v>46260161</x:v>
       </x:c>
       <x:c r="D70" s="0">
         <x:v>180000000</x:v>
@@ -3978,7 +3981,7 @@
         <x:v>2000000000</x:v>
       </x:c>
       <x:c r="F70" s="0">
-        <x:v>592056574</x:v>
+        <x:v>595217159</x:v>
       </x:c>
       <x:c r="G70" s="0">
         <x:v>2</x:v>
@@ -3987,13 +3990,13 @@
         <x:v>0.51</x:v>
       </x:c>
       <x:c r="I70" s="0">
-        <x:v>14.15</x:v>
+        <x:v>14.28</x:v>
       </x:c>
       <x:c r="J70" s="0">
-        <x:v>12.86</x:v>
+        <x:v>12.87</x:v>
       </x:c>
       <x:c r="K70" s="0" t="s">
-        <x:v>19</x:v>
+        <x:v>12</x:v>
       </x:c>
     </x:row>
     <x:row r="71" spans="1:11">
@@ -4004,7 +4007,7 @@
         <x:v>88</x:v>
       </x:c>
       <x:c r="C71" s="0">
-        <x:v>1814552</x:v>
+        <x:v>1914552</x:v>
       </x:c>
       <x:c r="D71" s="0">
         <x:v>25000000</x:v>
@@ -4013,22 +4016,22 @@
         <x:v>500000000</x:v>
       </x:c>
       <x:c r="F71" s="0">
-        <x:v>42596745</x:v>
+        <x:v>44957845</x:v>
       </x:c>
       <x:c r="G71" s="0">
         <x:v>4.84</x:v>
       </x:c>
       <x:c r="H71" s="0">
-        <x:v>0.35</x:v>
+        <x:v>0.37</x:v>
       </x:c>
       <x:c r="I71" s="0">
-        <x:v>23.72</x:v>
+        <x:v>24.1</x:v>
       </x:c>
       <x:c r="J71" s="0">
         <x:v>23.48</x:v>
       </x:c>
       <x:c r="K71" s="0" t="s">
-        <x:v>19</x:v>
+        <x:v>12</x:v>
       </x:c>
     </x:row>
     <x:row r="72" spans="1:11">
@@ -4057,13 +4060,13 @@
         <x:v>0.3</x:v>
       </x:c>
       <x:c r="I72" s="0">
-        <x:v>37.24</x:v>
+        <x:v>37.7</x:v>
       </x:c>
       <x:c r="J72" s="0">
         <x:v>37.46</x:v>
       </x:c>
       <x:c r="K72" s="0" t="s">
-        <x:v>19</x:v>
+        <x:v>22</x:v>
       </x:c>
     </x:row>
     <x:row r="73" spans="1:11">
@@ -4092,7 +4095,7 @@
         <x:v>1.42</x:v>
       </x:c>
       <x:c r="I73" s="0">
-        <x:v>127.8</x:v>
+        <x:v>129.5</x:v>
       </x:c>
       <x:c r="J73" s="0">
         <x:v>137.41</x:v>
@@ -4109,7 +4112,7 @@
         <x:v>100</x:v>
       </x:c>
       <x:c r="C74" s="0">
-        <x:v>110740</x:v>
+        <x:v>113000</x:v>
       </x:c>
       <x:c r="D74" s="0">
         <x:v>1000000</x:v>
@@ -4118,7 +4121,7 @@
         <x:v>300000000</x:v>
       </x:c>
       <x:c r="F74" s="0">
-        <x:v>31594890</x:v>
+        <x:v>32196680</x:v>
       </x:c>
       <x:c r="G74" s="0">
         <x:v>0.98</x:v>
@@ -4127,13 +4130,13 @@
         <x:v>0.11</x:v>
       </x:c>
       <x:c r="I74" s="0">
-        <x:v>274.5</x:v>
+        <x:v>280.5</x:v>
       </x:c>
       <x:c r="J74" s="0">
-        <x:v>285.31</x:v>
+        <x:v>284.93</x:v>
       </x:c>
       <x:c r="K74" s="0" t="s">
-        <x:v>19</x:v>
+        <x:v>12</x:v>
       </x:c>
     </x:row>
     <x:row r="75" spans="1:11">
@@ -4144,7 +4147,7 @@
         <x:v>100</x:v>
       </x:c>
       <x:c r="C75" s="0">
-        <x:v>975029</x:v>
+        <x:v>1033649</x:v>
       </x:c>
       <x:c r="D75" s="0">
         <x:v>2850000</x:v>
@@ -4153,22 +4156,22 @@
         <x:v>100000000</x:v>
       </x:c>
       <x:c r="F75" s="0">
-        <x:v>29677673</x:v>
+        <x:v>31466228</x:v>
       </x:c>
       <x:c r="G75" s="0">
         <x:v>2.41</x:v>
       </x:c>
       <x:c r="H75" s="0">
-        <x:v>0.82</x:v>
+        <x:v>0.87</x:v>
       </x:c>
       <x:c r="I75" s="0">
-        <x:v>30.6</x:v>
+        <x:v>30.4</x:v>
       </x:c>
       <x:c r="J75" s="0">
         <x:v>30.44</x:v>
       </x:c>
       <x:c r="K75" s="0" t="s">
-        <x:v>19</x:v>
+        <x:v>12</x:v>
       </x:c>
     </x:row>
     <x:row r="76" spans="1:11">
@@ -4197,7 +4200,7 @@
         <x:v>0.03</x:v>
       </x:c>
       <x:c r="I76" s="0">
-        <x:v>52.4</x:v>
+        <x:v>52.3</x:v>
       </x:c>
       <x:c r="J76" s="0">
         <x:v>53.69</x:v>
@@ -4232,7 +4235,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="I77" s="0">
-        <x:v>8.7</x:v>
+        <x:v>9.02</x:v>
       </x:c>
       <x:c r="J77" s="0">
         <x:v>0</x:v>
@@ -4264,7 +4267,7 @@
         <x:v>0.65</x:v>
       </x:c>
       <x:c r="I78" s="0">
-        <x:v>1.38</x:v>
+        <x:v>1.49</x:v>
       </x:c>
       <x:c r="J78" s="0">
         <x:v>4.89</x:v>
@@ -4281,7 +4284,7 @@
         <x:v>109</x:v>
       </x:c>
       <x:c r="C79" s="0">
-        <x:v>1285319</x:v>
+        <x:v>1365338</x:v>
       </x:c>
       <x:c r="D79" s="0">
         <x:v>36000000</x:v>
@@ -4290,22 +4293,22 @@
         <x:v>250000000</x:v>
       </x:c>
       <x:c r="F79" s="0">
-        <x:v>6947586</x:v>
+        <x:v>7376488</x:v>
       </x:c>
       <x:c r="G79" s="0">
         <x:v>3.75</x:v>
       </x:c>
       <x:c r="H79" s="0">
-        <x:v>0.13</x:v>
+        <x:v>0.14</x:v>
       </x:c>
       <x:c r="I79" s="0">
-        <x:v>5.41</x:v>
+        <x:v>5.53</x:v>
       </x:c>
       <x:c r="J79" s="0">
-        <x:v>5.41</x:v>
+        <x:v>5.4</x:v>
       </x:c>
       <x:c r="K79" s="0" t="s">
-        <x:v>19</x:v>
+        <x:v>12</x:v>
       </x:c>
     </x:row>
     <x:row r="80" spans="1:11">
@@ -4334,7 +4337,7 @@
         <x:v>0.32</x:v>
       </x:c>
       <x:c r="I80" s="0">
-        <x:v>7.23</x:v>
+        <x:v>7.34</x:v>
       </x:c>
       <x:c r="J80" s="0">
         <x:v>7.98</x:v>
@@ -4351,7 +4354,7 @@
         <x:v>113</x:v>
       </x:c>
       <x:c r="C81" s="0">
-        <x:v>6329227</x:v>
+        <x:v>6384227</x:v>
       </x:c>
       <x:c r="D81" s="0">
         <x:v>13500000</x:v>
@@ -4360,22 +4363,22 @@
         <x:v>400000000</x:v>
       </x:c>
       <x:c r="F81" s="0">
-        <x:v>102521068</x:v>
+        <x:v>103421418</x:v>
       </x:c>
       <x:c r="G81" s="0">
         <x:v>6.75</x:v>
       </x:c>
       <x:c r="H81" s="0">
-        <x:v>3.16</x:v>
+        <x:v>3.19</x:v>
       </x:c>
       <x:c r="I81" s="0">
-        <x:v>16.41</x:v>
+        <x:v>17.65</x:v>
       </x:c>
       <x:c r="J81" s="0">
         <x:v>16.2</x:v>
       </x:c>
       <x:c r="K81" s="0" t="s">
-        <x:v>19</x:v>
+        <x:v>12</x:v>
       </x:c>
     </x:row>
     <x:row r="82" spans="1:11">
@@ -4404,7 +4407,7 @@
         <x:v>3.86</x:v>
       </x:c>
       <x:c r="I82" s="0">
-        <x:v>5</x:v>
+        <x:v>5.13</x:v>
       </x:c>
       <x:c r="J82" s="0">
         <x:v>6.91</x:v>
@@ -4439,7 +4442,7 @@
         <x:v>0.71</x:v>
       </x:c>
       <x:c r="I83" s="0">
-        <x:v>5.62</x:v>
+        <x:v>6.18</x:v>
       </x:c>
       <x:c r="J83" s="0">
         <x:v>23.68</x:v>
@@ -4474,13 +4477,13 @@
         <x:v>1.07</x:v>
       </x:c>
       <x:c r="I84" s="0">
-        <x:v>4.03</x:v>
+        <x:v>3.66</x:v>
       </x:c>
       <x:c r="J84" s="0">
         <x:v>3.72</x:v>
       </x:c>
       <x:c r="K84" s="0" t="s">
-        <x:v>19</x:v>
+        <x:v>22</x:v>
       </x:c>
     </x:row>
     <x:row r="85" spans="1:11">
@@ -4509,7 +4512,7 @@
         <x:v>3.83</x:v>
       </x:c>
       <x:c r="I85" s="0">
-        <x:v>9.41</x:v>
+        <x:v>9.8</x:v>
       </x:c>
       <x:c r="J85" s="0">
         <x:v>0.76</x:v>
@@ -4579,7 +4582,7 @@
         <x:v>8.08</x:v>
       </x:c>
       <x:c r="I87" s="0">
-        <x:v>10.5</x:v>
+        <x:v>11.5</x:v>
       </x:c>
       <x:c r="J87" s="0">
         <x:v>0.73</x:v>
@@ -4614,13 +4617,13 @@
         <x:v>0.11</x:v>
       </x:c>
       <x:c r="I88" s="0">
-        <x:v>54.45</x:v>
+        <x:v>54.9</x:v>
       </x:c>
       <x:c r="J88" s="0">
         <x:v>60.51</x:v>
       </x:c>
       <x:c r="K88" s="0" t="s">
-        <x:v>19</x:v>
+        <x:v>22</x:v>
       </x:c>
     </x:row>
     <x:row r="89" spans="1:11">
@@ -4649,7 +4652,7 @@
         <x:v>0.19</x:v>
       </x:c>
       <x:c r="I89" s="0">
-        <x:v>0.98</x:v>
+        <x:v>1.03</x:v>
       </x:c>
       <x:c r="J89" s="0">
         <x:v>1.14</x:v>
@@ -4684,7 +4687,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="I90" s="0">
-        <x:v>118.6</x:v>
+        <x:v>119.5</x:v>
       </x:c>
       <x:c r="J90" s="0">
         <x:v>0</x:v>
@@ -4716,7 +4719,7 @@
         <x:v>0.01</x:v>
       </x:c>
       <x:c r="I91" s="0">
-        <x:v>3.3</x:v>
+        <x:v>3.41</x:v>
       </x:c>
       <x:c r="J91" s="0">
         <x:v>6.13</x:v>
@@ -4733,7 +4736,7 @@
         <x:v>134</x:v>
       </x:c>
       <x:c r="C92" s="0">
-        <x:v>11196031</x:v>
+        <x:v>12590031</x:v>
       </x:c>
       <x:c r="D92" s="0">
         <x:v>25000000</x:v>
@@ -4742,22 +4745,22 @@
         <x:v>240000000</x:v>
       </x:c>
       <x:c r="F92" s="0">
-        <x:v>110381015</x:v>
+        <x:v>123385085</x:v>
       </x:c>
       <x:c r="G92" s="0">
         <x:v>1.04</x:v>
       </x:c>
       <x:c r="H92" s="0">
-        <x:v>0.46</x:v>
+        <x:v>0.52</x:v>
       </x:c>
       <x:c r="I92" s="0">
-        <x:v>9.3</x:v>
+        <x:v>9.54</x:v>
       </x:c>
       <x:c r="J92" s="0">
-        <x:v>9.86</x:v>
+        <x:v>9.8</x:v>
       </x:c>
       <x:c r="K92" s="0" t="s">
-        <x:v>19</x:v>
+        <x:v>12</x:v>
       </x:c>
     </x:row>
     <x:row r="93" spans="1:11">
@@ -4786,7 +4789,7 @@
         <x:v>0.36</x:v>
       </x:c>
       <x:c r="I93" s="0">
-        <x:v>7.23</x:v>
+        <x:v>7.34</x:v>
       </x:c>
       <x:c r="J93" s="0">
         <x:v>9.69</x:v>
@@ -4821,7 +4824,7 @@
         <x:v>0.13</x:v>
       </x:c>
       <x:c r="I94" s="0">
-        <x:v>15.61</x:v>
+        <x:v>14.72</x:v>
       </x:c>
       <x:c r="J94" s="0">
         <x:v>15.28</x:v>
@@ -4856,7 +4859,7 @@
         <x:v>1.07</x:v>
       </x:c>
       <x:c r="I95" s="0">
-        <x:v>1.43</x:v>
+        <x:v>1.49</x:v>
       </x:c>
       <x:c r="J95" s="0">
         <x:v>1.51</x:v>
@@ -4891,7 +4894,7 @@
         <x:v>0.27</x:v>
       </x:c>
       <x:c r="I96" s="0">
-        <x:v>16.17</x:v>
+        <x:v>16.14</x:v>
       </x:c>
       <x:c r="J96" s="0">
         <x:v>15.9</x:v>
@@ -4908,7 +4911,7 @@
         <x:v>142</x:v>
       </x:c>
       <x:c r="C97" s="0">
-        <x:v>10092017</x:v>
+        <x:v>11514033</x:v>
       </x:c>
       <x:c r="D97" s="0">
         <x:v>40000000</x:v>
@@ -4917,22 +4920,22 @@
         <x:v>1000000000</x:v>
       </x:c>
       <x:c r="F97" s="0">
-        <x:v>174648368</x:v>
+        <x:v>199305477</x:v>
       </x:c>
       <x:c r="G97" s="0">
         <x:v>4.81</x:v>
       </x:c>
       <x:c r="H97" s="0">
-        <x:v>1.21</x:v>
+        <x:v>1.38</x:v>
       </x:c>
       <x:c r="I97" s="0">
-        <x:v>17.97</x:v>
+        <x:v>19.42</x:v>
       </x:c>
       <x:c r="J97" s="0">
         <x:v>17.31</x:v>
       </x:c>
       <x:c r="K97" s="0" t="s">
-        <x:v>19</x:v>
+        <x:v>12</x:v>
       </x:c>
     </x:row>
     <x:row r="98" spans="1:11">
@@ -4961,7 +4964,7 @@
         <x:v>0.86</x:v>
       </x:c>
       <x:c r="I98" s="0">
-        <x:v>3.41</x:v>
+        <x:v>3.4</x:v>
       </x:c>
       <x:c r="J98" s="0">
         <x:v>3.59</x:v>
@@ -4996,7 +4999,7 @@
         <x:v>0.21</x:v>
       </x:c>
       <x:c r="I99" s="0">
-        <x:v>401</x:v>
+        <x:v>402.75</x:v>
       </x:c>
       <x:c r="J99" s="0">
         <x:v>380.17</x:v>
@@ -5031,7 +5034,7 @@
         <x:v>1.59</x:v>
       </x:c>
       <x:c r="I100" s="0">
-        <x:v>57.5</x:v>
+        <x:v>57.45</x:v>
       </x:c>
       <x:c r="J100" s="0">
         <x:v>68.91</x:v>
@@ -5066,7 +5069,7 @@
         <x:v>0.67</x:v>
       </x:c>
       <x:c r="I101" s="0">
-        <x:v>23.8</x:v>
+        <x:v>26.18</x:v>
       </x:c>
       <x:c r="J101" s="0">
         <x:v>38.82</x:v>
@@ -5101,13 +5104,13 @@
         <x:v>2.4</x:v>
       </x:c>
       <x:c r="I102" s="0">
-        <x:v>42.24</x:v>
+        <x:v>43.9</x:v>
       </x:c>
       <x:c r="J102" s="0">
         <x:v>47.51</x:v>
       </x:c>
       <x:c r="K102" s="0" t="s">
-        <x:v>19</x:v>
+        <x:v>22</x:v>
       </x:c>
     </x:row>
     <x:row r="103" spans="1:11">
@@ -5136,7 +5139,7 @@
         <x:v>2.36</x:v>
       </x:c>
       <x:c r="I103" s="0">
-        <x:v>7.96</x:v>
+        <x:v>8.61</x:v>
       </x:c>
       <x:c r="J103" s="0">
         <x:v>32.87</x:v>
@@ -5171,7 +5174,7 @@
         <x:v>0.02</x:v>
       </x:c>
       <x:c r="I104" s="0">
-        <x:v>14</x:v>
+        <x:v>14.03</x:v>
       </x:c>
       <x:c r="J104" s="0">
         <x:v>13.65</x:v>
@@ -5206,7 +5209,7 @@
         <x:v>2.11</x:v>
       </x:c>
       <x:c r="I105" s="0">
-        <x:v>15.58</x:v>
+        <x:v>15.71</x:v>
       </x:c>
       <x:c r="J105" s="0">
         <x:v>21.09</x:v>
@@ -5223,7 +5226,7 @@
         <x:v>160</x:v>
       </x:c>
       <x:c r="C106" s="0">
-        <x:v>1423000</x:v>
+        <x:v>1618000</x:v>
       </x:c>
       <x:c r="D106" s="0">
         <x:v>21739600</x:v>
@@ -5232,22 +5235,22 @@
         <x:v>350000000</x:v>
       </x:c>
       <x:c r="F106" s="0">
-        <x:v>11563775</x:v>
+        <x:v>13007224</x:v>
       </x:c>
       <x:c r="G106" s="0">
         <x:v>2</x:v>
       </x:c>
       <x:c r="H106" s="0">
-        <x:v>0.13</x:v>
+        <x:v>0.15</x:v>
       </x:c>
       <x:c r="I106" s="0">
-        <x:v>7.57</x:v>
+        <x:v>7.69</x:v>
       </x:c>
       <x:c r="J106" s="0">
-        <x:v>8.13</x:v>
+        <x:v>8.04</x:v>
       </x:c>
       <x:c r="K106" s="0" t="s">
-        <x:v>16</x:v>
+        <x:v>12</x:v>
       </x:c>
     </x:row>
     <x:row r="107" spans="1:11">
@@ -5276,7 +5279,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="I107" s="0">
-        <x:v>8.78</x:v>
+        <x:v>8.9</x:v>
       </x:c>
       <x:c r="J107" s="0">
         <x:v>0</x:v>
@@ -5308,7 +5311,7 @@
         <x:v>0.57</x:v>
       </x:c>
       <x:c r="I108" s="0">
-        <x:v>7.65</x:v>
+        <x:v>7.67</x:v>
       </x:c>
       <x:c r="J108" s="0">
         <x:v>6.98</x:v>
@@ -5343,7 +5346,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="I109" s="0">
-        <x:v>127.8</x:v>
+        <x:v>129.5</x:v>
       </x:c>
       <x:c r="J109" s="0">
         <x:v>0</x:v>
@@ -5375,7 +5378,7 @@
         <x:v>0.64</x:v>
       </x:c>
       <x:c r="I110" s="0">
-        <x:v>15.34</x:v>
+        <x:v>16.87</x:v>
       </x:c>
       <x:c r="J110" s="0">
         <x:v>7.61</x:v>
@@ -5410,7 +5413,7 @@
         <x:v>0.18</x:v>
       </x:c>
       <x:c r="I111" s="0">
-        <x:v>19.87</x:v>
+        <x:v>20.24</x:v>
       </x:c>
       <x:c r="J111" s="0">
         <x:v>28.89</x:v>
@@ -5445,7 +5448,7 @@
         <x:v>1.62</x:v>
       </x:c>
       <x:c r="I112" s="0">
-        <x:v>8.05</x:v>
+        <x:v>8.11</x:v>
       </x:c>
       <x:c r="J112" s="0">
         <x:v>9.52</x:v>
@@ -5480,7 +5483,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="I113" s="0">
-        <x:v>4.15</x:v>
+        <x:v>4.12</x:v>
       </x:c>
       <x:c r="J113" s="0">
         <x:v>0</x:v>
@@ -5512,7 +5515,7 @@
         <x:v>2.79</x:v>
       </x:c>
       <x:c r="I114" s="0">
-        <x:v>21.06</x:v>
+        <x:v>21.02</x:v>
       </x:c>
       <x:c r="J114" s="0">
         <x:v>23.25</x:v>
@@ -5547,7 +5550,7 @@
         <x:v>1.13</x:v>
       </x:c>
       <x:c r="I115" s="0">
-        <x:v>48.02</x:v>
+        <x:v>48.38</x:v>
       </x:c>
       <x:c r="J115" s="0">
         <x:v>28.18</x:v>
@@ -5582,7 +5585,7 @@
         <x:v>0.78</x:v>
       </x:c>
       <x:c r="I116" s="0">
-        <x:v>9.3</x:v>
+        <x:v>9.24</x:v>
       </x:c>
       <x:c r="J116" s="0">
         <x:v>13.34</x:v>
@@ -5617,7 +5620,7 @@
         <x:v>0.71</x:v>
       </x:c>
       <x:c r="I117" s="0">
-        <x:v>28.72</x:v>
+        <x:v>27.4</x:v>
       </x:c>
       <x:c r="J117" s="0">
         <x:v>39.18</x:v>
@@ -5652,7 +5655,7 @@
         <x:v>0.82</x:v>
       </x:c>
       <x:c r="I118" s="0">
-        <x:v>53.3</x:v>
+        <x:v>53.7</x:v>
       </x:c>
       <x:c r="J118" s="0">
         <x:v>59.93</x:v>
@@ -5687,7 +5690,7 @@
         <x:v>0.6</x:v>
       </x:c>
       <x:c r="I119" s="0">
-        <x:v>3.61</x:v>
+        <x:v>3.73</x:v>
       </x:c>
       <x:c r="J119" s="0">
         <x:v>48.39</x:v>
@@ -5722,7 +5725,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="I120" s="0">
-        <x:v>1.93</x:v>
+        <x:v>2.08</x:v>
       </x:c>
       <x:c r="J120" s="0">
         <x:v>0</x:v>
@@ -5754,7 +5757,7 @@
         <x:v>1.03</x:v>
       </x:c>
       <x:c r="I121" s="0">
-        <x:v>8.37</x:v>
+        <x:v>8.85</x:v>
       </x:c>
       <x:c r="J121" s="0">
         <x:v>26.19</x:v>
@@ -5771,7 +5774,7 @@
         <x:v>193</x:v>
       </x:c>
       <x:c r="C122" s="0">
-        <x:v>29146645</x:v>
+        <x:v>29346645</x:v>
       </x:c>
       <x:c r="D122" s="0">
         <x:v>35000000</x:v>
@@ -5780,22 +5783,22 @@
         <x:v>300000000</x:v>
       </x:c>
       <x:c r="F122" s="0">
-        <x:v>229749719</x:v>
+        <x:v>230894719</x:v>
       </x:c>
       <x:c r="G122" s="0">
         <x:v>16.25</x:v>
       </x:c>
       <x:c r="H122" s="0">
-        <x:v>7.29</x:v>
+        <x:v>7.34</x:v>
       </x:c>
       <x:c r="I122" s="0">
-        <x:v>5.82</x:v>
+        <x:v>5.55</x:v>
       </x:c>
       <x:c r="J122" s="0">
-        <x:v>7.88</x:v>
+        <x:v>7.87</x:v>
       </x:c>
       <x:c r="K122" s="0" t="s">
-        <x:v>15</x:v>
+        <x:v>12</x:v>
       </x:c>
     </x:row>
     <x:row r="123" spans="1:11">
@@ -5824,7 +5827,7 @@
         <x:v>0.18</x:v>
       </x:c>
       <x:c r="I123" s="0">
-        <x:v>29.98</x:v>
+        <x:v>30.2</x:v>
       </x:c>
       <x:c r="J123" s="0">
         <x:v>61.87</x:v>
@@ -5859,7 +5862,7 @@
         <x:v>0.29</x:v>
       </x:c>
       <x:c r="I124" s="0">
-        <x:v>13.99</x:v>
+        <x:v>14.34</x:v>
       </x:c>
       <x:c r="J124" s="0">
         <x:v>21.06</x:v>
@@ -5894,7 +5897,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="I125" s="0">
-        <x:v>3.61</x:v>
+        <x:v>3.73</x:v>
       </x:c>
       <x:c r="J125" s="0">
         <x:v>0</x:v>
@@ -5926,7 +5929,7 @@
         <x:v>1.17</x:v>
       </x:c>
       <x:c r="I126" s="0">
-        <x:v>14.15</x:v>
+        <x:v>14.28</x:v>
       </x:c>
       <x:c r="J126" s="0">
         <x:v>9.8</x:v>
@@ -5961,7 +5964,7 @@
         <x:v>3.29</x:v>
       </x:c>
       <x:c r="I127" s="0">
-        <x:v>14.8</x:v>
+        <x:v>16.28</x:v>
       </x:c>
       <x:c r="J127" s="0">
         <x:v>23.95</x:v>
@@ -5996,7 +5999,7 @@
         <x:v>0.09</x:v>
       </x:c>
       <x:c r="I128" s="0">
-        <x:v>401</x:v>
+        <x:v>402.75</x:v>
       </x:c>
       <x:c r="J128" s="0">
         <x:v>528.86</x:v>
@@ -6031,7 +6034,7 @@
         <x:v>0.94</x:v>
       </x:c>
       <x:c r="I129" s="0">
-        <x:v>48.02</x:v>
+        <x:v>48.38</x:v>
       </x:c>
       <x:c r="J129" s="0">
         <x:v>24.19</x:v>
@@ -6066,7 +6069,7 @@
         <x:v>0.52</x:v>
       </x:c>
       <x:c r="I130" s="0">
-        <x:v>14.15</x:v>
+        <x:v>14.28</x:v>
       </x:c>
       <x:c r="J130" s="0">
         <x:v>10.74</x:v>
@@ -6101,7 +6104,7 @@
         <x:v>0.69</x:v>
       </x:c>
       <x:c r="I131" s="0">
-        <x:v>5.41</x:v>
+        <x:v>5.53</x:v>
       </x:c>
       <x:c r="J131" s="0">
         <x:v>6.01</x:v>
@@ -6136,7 +6139,7 @@
         <x:v>2.15</x:v>
       </x:c>
       <x:c r="I132" s="0">
-        <x:v>10.69</x:v>
+        <x:v>11.03</x:v>
       </x:c>
       <x:c r="J132" s="0">
         <x:v>20.61</x:v>
@@ -6171,7 +6174,7 @@
         <x:v>0.1</x:v>
       </x:c>
       <x:c r="I133" s="0">
-        <x:v>4.07</x:v>
+        <x:v>4.34</x:v>
       </x:c>
       <x:c r="J133" s="0">
         <x:v>4.46</x:v>
@@ -6206,7 +6209,7 @@
         <x:v>0.04</x:v>
       </x:c>
       <x:c r="I134" s="0">
-        <x:v>5</x:v>
+        <x:v>5.13</x:v>
       </x:c>
       <x:c r="J134" s="0">
         <x:v>12.82</x:v>
@@ -6241,7 +6244,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="I135" s="0">
-        <x:v>19.29</x:v>
+        <x:v>19.07</x:v>
       </x:c>
       <x:c r="J135" s="0">
         <x:v>0</x:v>
@@ -6273,7 +6276,7 @@
         <x:v>0.83</x:v>
       </x:c>
       <x:c r="I136" s="0">
-        <x:v>1.74</x:v>
+        <x:v>1.91</x:v>
       </x:c>
       <x:c r="J136" s="0">
         <x:v>52.14</x:v>
@@ -6308,7 +6311,7 @@
         <x:v>1.83</x:v>
       </x:c>
       <x:c r="I137" s="0">
-        <x:v>37.24</x:v>
+        <x:v>37.7</x:v>
       </x:c>
       <x:c r="J137" s="0">
         <x:v>39.62</x:v>
@@ -6325,7 +6328,7 @@
         <x:v>225</x:v>
       </x:c>
       <x:c r="C138" s="0">
-        <x:v>5899828</x:v>
+        <x:v>5999828</x:v>
       </x:c>
       <x:c r="D138" s="0">
         <x:v>3000000</x:v>
@@ -6334,22 +6337,22 @@
         <x:v>300000000</x:v>
       </x:c>
       <x:c r="F138" s="0">
-        <x:v>223937644</x:v>
+        <x:v>226137644</x:v>
       </x:c>
       <x:c r="G138" s="0">
         <x:v>3.75</x:v>
       </x:c>
       <x:c r="H138" s="0">
-        <x:v>1.47</x:v>
+        <x:v>1.5</x:v>
       </x:c>
       <x:c r="I138" s="0">
-        <x:v>22.7</x:v>
+        <x:v>23.16</x:v>
       </x:c>
       <x:c r="J138" s="0">
-        <x:v>37.96</x:v>
+        <x:v>37.69</x:v>
       </x:c>
       <x:c r="K138" s="0" t="s">
-        <x:v>30</x:v>
+        <x:v>12</x:v>
       </x:c>
     </x:row>
     <x:row r="139" spans="1:11">
@@ -6378,7 +6381,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="I139" s="0">
-        <x:v>18.01</x:v>
+        <x:v>18.39</x:v>
       </x:c>
       <x:c r="J139" s="0">
         <x:v>0</x:v>
@@ -6392,7 +6395,7 @@
         <x:v>227</x:v>
       </x:c>
       <x:c r="C140" s="0">
-        <x:v>14837681</x:v>
+        <x:v>15837681</x:v>
       </x:c>
       <x:c r="D140" s="0">
         <x:v>6500000</x:v>
@@ -6401,22 +6404,22 @@
         <x:v>100000000</x:v>
       </x:c>
       <x:c r="F140" s="0">
-        <x:v>53535183</x:v>
+        <x:v>56135183</x:v>
       </x:c>
       <x:c r="G140" s="0">
-        <x:v>1.43</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="H140" s="0">
-        <x:v>0.59</x:v>
+        <x:v>0.63</x:v>
       </x:c>
       <x:c r="I140" s="0">
-        <x:v>2.63</x:v>
+        <x:v>2.59</x:v>
       </x:c>
       <x:c r="J140" s="0">
-        <x:v>3.61</x:v>
+        <x:v>3.54</x:v>
       </x:c>
       <x:c r="K140" s="0" t="s">
-        <x:v>27</x:v>
+        <x:v>12</x:v>
       </x:c>
     </x:row>
     <x:row r="141" spans="1:11">
@@ -6445,7 +6448,7 @@
         <x:v>0.37</x:v>
       </x:c>
       <x:c r="I141" s="0">
-        <x:v>29.3</x:v>
+        <x:v>29.62</x:v>
       </x:c>
       <x:c r="J141" s="0">
         <x:v>30.83</x:v>
@@ -6480,7 +6483,7 @@
         <x:v>0.1</x:v>
       </x:c>
       <x:c r="I142" s="0">
-        <x:v>284.25</x:v>
+        <x:v>287.5</x:v>
       </x:c>
       <x:c r="J142" s="0">
         <x:v>299.91</x:v>
@@ -6515,7 +6518,7 @@
         <x:v>0.03</x:v>
       </x:c>
       <x:c r="I143" s="0">
-        <x:v>19.61</x:v>
+        <x:v>19.85</x:v>
       </x:c>
       <x:c r="J143" s="0">
         <x:v>19.3</x:v>
@@ -6550,7 +6553,7 @@
         <x:v>0.54</x:v>
       </x:c>
       <x:c r="I144" s="0">
-        <x:v>243.5</x:v>
+        <x:v>236.1</x:v>
       </x:c>
       <x:c r="J144" s="0">
         <x:v>83</x:v>
@@ -6585,7 +6588,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="I145" s="0">
-        <x:v>23.52</x:v>
+        <x:v>23.6</x:v>
       </x:c>
       <x:c r="J145" s="0">
         <x:v>40.97</x:v>
@@ -6620,7 +6623,7 @@
         <x:v>0.62</x:v>
       </x:c>
       <x:c r="I146" s="0">
-        <x:v>5.62</x:v>
+        <x:v>6.18</x:v>
       </x:c>
       <x:c r="J146" s="0">
         <x:v>23.68</x:v>
@@ -6655,7 +6658,7 @@
         <x:v>0.08</x:v>
       </x:c>
       <x:c r="I147" s="0">
-        <x:v>14</x:v>
+        <x:v>14.03</x:v>
       </x:c>
       <x:c r="J147" s="0">
         <x:v>5.49</x:v>
@@ -6690,7 +6693,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="I148" s="0">
-        <x:v>16.17</x:v>
+        <x:v>16.14</x:v>
       </x:c>
       <x:c r="J148" s="0">
         <x:v>0</x:v>
@@ -6722,7 +6725,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="I149" s="0">
-        <x:v>4.36</x:v>
+        <x:v>4.42</x:v>
       </x:c>
       <x:c r="J149" s="0">
         <x:v>0</x:v>
@@ -6754,7 +6757,7 @@
         <x:v>0.33</x:v>
       </x:c>
       <x:c r="I150" s="0">
-        <x:v>1.88</x:v>
+        <x:v>1.93</x:v>
       </x:c>
       <x:c r="J150" s="0">
         <x:v>3.98</x:v>
@@ -6789,7 +6792,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I151" s="0">
-        <x:v>5.61</x:v>
+        <x:v>5.64</x:v>
       </x:c>
       <x:c r="J151" s="0">
         <x:v>6.6</x:v>
@@ -6824,7 +6827,7 @@
         <x:v>0.33</x:v>
       </x:c>
       <x:c r="I152" s="0">
-        <x:v>10.69</x:v>
+        <x:v>11.03</x:v>
       </x:c>
       <x:c r="J152" s="0">
         <x:v>17.83</x:v>
@@ -6859,7 +6862,7 @@
         <x:v>0.03</x:v>
       </x:c>
       <x:c r="I153" s="0">
-        <x:v>24.58</x:v>
+        <x:v>24.4</x:v>
       </x:c>
       <x:c r="J153" s="0">
         <x:v>38.06</x:v>
@@ -6894,7 +6897,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="I154" s="0">
-        <x:v>207.4</x:v>
+        <x:v>213.8</x:v>
       </x:c>
       <x:c r="J154" s="0">
         <x:v>0</x:v>
@@ -6926,7 +6929,7 @@
         <x:v>0.86</x:v>
       </x:c>
       <x:c r="I155" s="0">
-        <x:v>25.8</x:v>
+        <x:v>26.9</x:v>
       </x:c>
       <x:c r="J155" s="0">
         <x:v>41.13</x:v>
@@ -6961,7 +6964,7 @@
         <x:v>0.04</x:v>
       </x:c>
       <x:c r="I156" s="0">
-        <x:v>2.92</x:v>
+        <x:v>3.03</x:v>
       </x:c>
       <x:c r="J156" s="0">
         <x:v>20.11</x:v>
@@ -6996,7 +6999,7 @@
         <x:v>0.04</x:v>
       </x:c>
       <x:c r="I157" s="0">
-        <x:v>3.66</x:v>
+        <x:v>3.64</x:v>
       </x:c>
       <x:c r="J157" s="0">
         <x:v>39.43</x:v>
@@ -7031,7 +7034,7 @@
         <x:v>0.12</x:v>
       </x:c>
       <x:c r="I158" s="0">
-        <x:v>18.37</x:v>
+        <x:v>18.66</x:v>
       </x:c>
       <x:c r="J158" s="0">
         <x:v>16.34</x:v>
@@ -7066,7 +7069,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="I159" s="0">
-        <x:v>9.55</x:v>
+        <x:v>9.72</x:v>
       </x:c>
       <x:c r="J159" s="0">
         <x:v>0</x:v>
@@ -7098,7 +7101,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="I160" s="0">
-        <x:v>39.02</x:v>
+        <x:v>39.16</x:v>
       </x:c>
       <x:c r="J160" s="0">
         <x:v>0</x:v>
@@ -7130,7 +7133,7 @@
         <x:v>0.6</x:v>
       </x:c>
       <x:c r="I161" s="0">
-        <x:v>14.28</x:v>
+        <x:v>12.86</x:v>
       </x:c>
       <x:c r="J161" s="0">
         <x:v>38.88</x:v>
@@ -7165,7 +7168,7 @@
         <x:v>0.1</x:v>
       </x:c>
       <x:c r="I162" s="0">
-        <x:v>4.25</x:v>
+        <x:v>4.67</x:v>
       </x:c>
       <x:c r="J162" s="0">
         <x:v>10.75</x:v>
@@ -7200,7 +7203,7 @@
         <x:v>2.16</x:v>
       </x:c>
       <x:c r="I163" s="0">
-        <x:v>28.3</x:v>
+        <x:v>29.88</x:v>
       </x:c>
       <x:c r="J163" s="0">
         <x:v>37.66</x:v>
@@ -7235,7 +7238,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="I164" s="0">
-        <x:v>1.49</x:v>
+        <x:v>1.63</x:v>
       </x:c>
       <x:c r="J164" s="0">
         <x:v>0</x:v>
@@ -7267,7 +7270,7 @@
         <x:v>0.4</x:v>
       </x:c>
       <x:c r="I165" s="0">
-        <x:v>7.23</x:v>
+        <x:v>7.34</x:v>
       </x:c>
       <x:c r="J165" s="0">
         <x:v>15.68</x:v>
@@ -7302,7 +7305,7 @@
         <x:v>0.15</x:v>
       </x:c>
       <x:c r="I166" s="0">
-        <x:v>1.33</x:v>
+        <x:v>1.37</x:v>
       </x:c>
       <x:c r="J166" s="0">
         <x:v>4.02</x:v>
@@ -7337,7 +7340,7 @@
         <x:v>0.01</x:v>
       </x:c>
       <x:c r="I167" s="0">
-        <x:v>4.25</x:v>
+        <x:v>4.67</x:v>
       </x:c>
       <x:c r="J167" s="0">
         <x:v>161.23</x:v>
@@ -7372,7 +7375,7 @@
         <x:v>1.25</x:v>
       </x:c>
       <x:c r="I168" s="0">
-        <x:v>1.63</x:v>
+        <x:v>1.73</x:v>
       </x:c>
       <x:c r="J168" s="0">
         <x:v>4.93</x:v>
@@ -7407,7 +7410,7 @@
         <x:v>0.1</x:v>
       </x:c>
       <x:c r="I169" s="0">
-        <x:v>100.2</x:v>
+        <x:v>98.55</x:v>
       </x:c>
       <x:c r="J169" s="0">
         <x:v>95.58</x:v>
@@ -7442,7 +7445,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="I170" s="0">
-        <x:v>43.92</x:v>
+        <x:v>43.88</x:v>
       </x:c>
       <x:c r="J170" s="0">
         <x:v>0</x:v>
@@ -7474,7 +7477,7 @@
         <x:v>1.31</x:v>
       </x:c>
       <x:c r="I171" s="0">
-        <x:v>2.4</x:v>
+        <x:v>2.46</x:v>
       </x:c>
       <x:c r="J171" s="0">
         <x:v>2.45</x:v>
@@ -7509,7 +7512,7 @@
         <x:v>1.08</x:v>
       </x:c>
       <x:c r="I172" s="0">
-        <x:v>54.45</x:v>
+        <x:v>54.9</x:v>
       </x:c>
       <x:c r="J172" s="0">
         <x:v>58.33</x:v>
@@ -7544,7 +7547,7 @@
         <x:v>2.11</x:v>
       </x:c>
       <x:c r="I173" s="0">
-        <x:v>15.58</x:v>
+        <x:v>15.71</x:v>
       </x:c>
       <x:c r="J173" s="0">
         <x:v>21.09</x:v>
@@ -7579,7 +7582,7 @@
         <x:v>0.19</x:v>
       </x:c>
       <x:c r="I174" s="0">
-        <x:v>3.75</x:v>
+        <x:v>3.81</x:v>
       </x:c>
       <x:c r="J174" s="0">
         <x:v>16.87</x:v>
@@ -7614,7 +7617,7 @@
         <x:v>0.18</x:v>
       </x:c>
       <x:c r="I175" s="0">
-        <x:v>3.3</x:v>
+        <x:v>3.41</x:v>
       </x:c>
       <x:c r="J175" s="0">
         <x:v>11.99</x:v>
@@ -7649,7 +7652,7 @@
         <x:v>0.68</x:v>
       </x:c>
       <x:c r="I176" s="0">
-        <x:v>12.12</x:v>
+        <x:v>13.33</x:v>
       </x:c>
       <x:c r="J176" s="0">
         <x:v>35.38</x:v>
@@ -7684,7 +7687,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="I177" s="0">
-        <x:v>5.38</x:v>
+        <x:v>5.45</x:v>
       </x:c>
       <x:c r="J177" s="0">
         <x:v>0</x:v>
@@ -7716,7 +7719,7 @@
         <x:v>0.27</x:v>
       </x:c>
       <x:c r="I178" s="0">
-        <x:v>4.12</x:v>
+        <x:v>4.53</x:v>
       </x:c>
       <x:c r="J178" s="0">
         <x:v>19.79</x:v>
@@ -7751,7 +7754,7 @@
         <x:v>0.06</x:v>
       </x:c>
       <x:c r="I179" s="0">
-        <x:v>10.47</x:v>
+        <x:v>10.3</x:v>
       </x:c>
       <x:c r="J179" s="0">
         <x:v>13.15</x:v>
@@ -7786,7 +7789,7 @@
         <x:v>3.45</x:v>
       </x:c>
       <x:c r="I180" s="0">
-        <x:v>1.43</x:v>
+        <x:v>1.49</x:v>
       </x:c>
       <x:c r="J180" s="0">
         <x:v>4.03</x:v>
@@ -7821,7 +7824,7 @@
         <x:v>0.15</x:v>
       </x:c>
       <x:c r="I181" s="0">
-        <x:v>3.35</x:v>
+        <x:v>3.55</x:v>
       </x:c>
       <x:c r="J181" s="0">
         <x:v>38.02</x:v>
@@ -7856,7 +7859,7 @@
         <x:v>4.31</x:v>
       </x:c>
       <x:c r="I182" s="0">
-        <x:v>30.6</x:v>
+        <x:v>30.4</x:v>
       </x:c>
       <x:c r="J182" s="0">
         <x:v>17.65</x:v>
@@ -7891,7 +7894,7 @@
         <x:v>0.1</x:v>
       </x:c>
       <x:c r="I183" s="0">
-        <x:v>8.76</x:v>
+        <x:v>9.57</x:v>
       </x:c>
       <x:c r="J183" s="0">
         <x:v>68.15</x:v>
@@ -7926,7 +7929,7 @@
         <x:v>0.92</x:v>
       </x:c>
       <x:c r="I184" s="0">
-        <x:v>9.58</x:v>
+        <x:v>9.77</x:v>
       </x:c>
       <x:c r="J184" s="0">
         <x:v>10.98</x:v>
@@ -7961,7 +7964,7 @@
         <x:v>0.16</x:v>
       </x:c>
       <x:c r="I185" s="0">
-        <x:v>16.98</x:v>
+        <x:v>17.83</x:v>
       </x:c>
       <x:c r="J185" s="0">
         <x:v>22.05</x:v>
@@ -7996,7 +7999,7 @@
         <x:v>0.8</x:v>
       </x:c>
       <x:c r="I186" s="0">
-        <x:v>121.5</x:v>
+        <x:v>122</x:v>
       </x:c>
       <x:c r="J186" s="0">
         <x:v>284.58</x:v>
@@ -8031,7 +8034,7 @@
         <x:v>1.67</x:v>
       </x:c>
       <x:c r="I187" s="0">
-        <x:v>41.7</x:v>
+        <x:v>37.54</x:v>
       </x:c>
       <x:c r="J187" s="0">
         <x:v>83.62</x:v>
@@ -8066,7 +8069,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="I188" s="0">
-        <x:v>8.88</x:v>
+        <x:v>8.79</x:v>
       </x:c>
       <x:c r="J188" s="0">
         <x:v>0</x:v>
@@ -8098,7 +8101,7 @@
         <x:v>0.33</x:v>
       </x:c>
       <x:c r="I189" s="0">
-        <x:v>13.27</x:v>
+        <x:v>13.66</x:v>
       </x:c>
       <x:c r="J189" s="0">
         <x:v>16.42</x:v>
@@ -8133,7 +8136,7 @@
         <x:v>0.02</x:v>
       </x:c>
       <x:c r="I190" s="0">
-        <x:v>3.95</x:v>
+        <x:v>4.04</x:v>
       </x:c>
       <x:c r="J190" s="0">
         <x:v>40.97</x:v>
@@ -8168,7 +8171,7 @@
         <x:v>0.29</x:v>
       </x:c>
       <x:c r="I191" s="0">
-        <x:v>8.7</x:v>
+        <x:v>9.02</x:v>
       </x:c>
       <x:c r="J191" s="0">
         <x:v>15.92</x:v>
@@ -8203,7 +8206,7 @@
         <x:v>3.13</x:v>
       </x:c>
       <x:c r="I192" s="0">
-        <x:v>108.3</x:v>
+        <x:v>109</x:v>
       </x:c>
       <x:c r="J192" s="0">
         <x:v>94.36</x:v>
@@ -8238,13 +8241,13 @@
         <x:v>5.26</x:v>
       </x:c>
       <x:c r="I193" s="0">
-        <x:v>4.26</x:v>
+        <x:v>4.32</x:v>
       </x:c>
       <x:c r="J193" s="0">
         <x:v>4.64</x:v>
       </x:c>
       <x:c r="K193" s="0" t="s">
-        <x:v>19</x:v>
+        <x:v>22</x:v>
       </x:c>
     </x:row>
     <x:row r="194" spans="1:11">
@@ -8273,7 +8276,7 @@
         <x:v>0.08</x:v>
       </x:c>
       <x:c r="I194" s="0">
-        <x:v>401</x:v>
+        <x:v>402.75</x:v>
       </x:c>
       <x:c r="J194" s="0">
         <x:v>429.82</x:v>
@@ -8308,7 +8311,7 @@
         <x:v>0.05</x:v>
       </x:c>
       <x:c r="I195" s="0">
-        <x:v>1.94</x:v>
+        <x:v>2.01</x:v>
       </x:c>
       <x:c r="J195" s="0">
         <x:v>2.64</x:v>
@@ -8343,7 +8346,7 @@
         <x:v>1.45</x:v>
       </x:c>
       <x:c r="I196" s="0">
-        <x:v>11.54</x:v>
+        <x:v>11.72</x:v>
       </x:c>
       <x:c r="J196" s="0">
         <x:v>8.23</x:v>
@@ -8378,7 +8381,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="I197" s="0">
-        <x:v>2.37</x:v>
+        <x:v>2.6</x:v>
       </x:c>
       <x:c r="J197" s="0">
         <x:v>0</x:v>
@@ -8410,7 +8413,7 @@
         <x:v>0.23</x:v>
       </x:c>
       <x:c r="I198" s="0">
-        <x:v>21.92</x:v>
+        <x:v>22.7</x:v>
       </x:c>
       <x:c r="J198" s="0">
         <x:v>23.66</x:v>
@@ -8445,7 +8448,7 @@
         <x:v>0.53</x:v>
       </x:c>
       <x:c r="I199" s="0">
-        <x:v>1.75</x:v>
+        <x:v>1.8</x:v>
       </x:c>
       <x:c r="J199" s="0">
         <x:v>5.03</x:v>
@@ -8480,7 +8483,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="I200" s="0">
-        <x:v>1.7</x:v>
+        <x:v>1.76</x:v>
       </x:c>
       <x:c r="J200" s="0">
         <x:v>0</x:v>
@@ -8544,7 +8547,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="I202" s="0">
-        <x:v>4.11</x:v>
+        <x:v>4.52</x:v>
       </x:c>
       <x:c r="J202" s="0">
         <x:v>0</x:v>
@@ -8576,7 +8579,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="I203" s="0">
-        <x:v>147</x:v>
+        <x:v>146.1</x:v>
       </x:c>
       <x:c r="J203" s="0">
         <x:v>50.97</x:v>
@@ -8611,7 +8614,7 @@
         <x:v>5.91</x:v>
       </x:c>
       <x:c r="I204" s="0">
-        <x:v>16.17</x:v>
+        <x:v>16.14</x:v>
       </x:c>
       <x:c r="J204" s="0">
         <x:v>10.93</x:v>
@@ -8646,7 +8649,7 @@
         <x:v>0.91</x:v>
       </x:c>
       <x:c r="I205" s="0">
-        <x:v>32.7</x:v>
+        <x:v>32.2</x:v>
       </x:c>
       <x:c r="J205" s="0">
         <x:v>38.14</x:v>
@@ -8681,7 +8684,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="I206" s="0">
-        <x:v>519.5</x:v>
+        <x:v>520</x:v>
       </x:c>
       <x:c r="J206" s="0">
         <x:v>0</x:v>
@@ -8713,7 +8716,7 @@
         <x:v>0.78</x:v>
       </x:c>
       <x:c r="I207" s="0">
-        <x:v>33.66</x:v>
+        <x:v>33.9</x:v>
       </x:c>
       <x:c r="J207" s="0">
         <x:v>25.82</x:v>
@@ -8748,7 +8751,7 @@
         <x:v>0.04</x:v>
       </x:c>
       <x:c r="I208" s="0">
-        <x:v>4.41</x:v>
+        <x:v>4.63</x:v>
       </x:c>
       <x:c r="J208" s="0">
         <x:v>4.56</x:v>
@@ -8783,7 +8786,7 @@
         <x:v>0.05</x:v>
       </x:c>
       <x:c r="I209" s="0">
-        <x:v>127.8</x:v>
+        <x:v>129.5</x:v>
       </x:c>
       <x:c r="J209" s="0">
         <x:v>31.92</x:v>
@@ -8818,7 +8821,7 @@
         <x:v>1.9</x:v>
       </x:c>
       <x:c r="I210" s="0">
-        <x:v>12.12</x:v>
+        <x:v>12.52</x:v>
       </x:c>
       <x:c r="J210" s="0">
         <x:v>15.2</x:v>
@@ -8853,7 +8856,7 @@
         <x:v>0.5</x:v>
       </x:c>
       <x:c r="I211" s="0">
-        <x:v>48.02</x:v>
+        <x:v>48.38</x:v>
       </x:c>
       <x:c r="J211" s="0">
         <x:v>20.53</x:v>
@@ -8888,7 +8891,7 @@
         <x:v>1.24</x:v>
       </x:c>
       <x:c r="I212" s="0">
-        <x:v>14.15</x:v>
+        <x:v>14.28</x:v>
       </x:c>
       <x:c r="J212" s="0">
         <x:v>4.48</x:v>
@@ -8923,7 +8926,7 @@
         <x:v>1.17</x:v>
       </x:c>
       <x:c r="I213" s="0">
-        <x:v>123.8</x:v>
+        <x:v>123.3</x:v>
       </x:c>
       <x:c r="J213" s="0">
         <x:v>39.56</x:v>
@@ -8958,7 +8961,7 @@
         <x:v>0.3</x:v>
       </x:c>
       <x:c r="I214" s="0">
-        <x:v>19.38</x:v>
+        <x:v>19.93</x:v>
       </x:c>
       <x:c r="J214" s="0">
         <x:v>15.05</x:v>
@@ -8975,7 +8978,7 @@
         <x:v>334</x:v>
       </x:c>
       <x:c r="C215" s="0">
-        <x:v>11323189</x:v>
+        <x:v>11348189</x:v>
       </x:c>
       <x:c r="D215" s="0">
         <x:v>21600000</x:v>
@@ -8984,22 +8987,22 @@
         <x:v>1200000000</x:v>
       </x:c>
       <x:c r="F215" s="0">
-        <x:v>186810680</x:v>
+        <x:v>187078430</x:v>
       </x:c>
       <x:c r="G215" s="0">
         <x:v>10</x:v>
       </x:c>
       <x:c r="H215" s="0">
-        <x:v>5.24</x:v>
+        <x:v>5.25</x:v>
       </x:c>
       <x:c r="I215" s="0">
-        <x:v>10.79</x:v>
+        <x:v>11.13</x:v>
       </x:c>
       <x:c r="J215" s="0">
-        <x:v>16.5</x:v>
+        <x:v>16.49</x:v>
       </x:c>
       <x:c r="K215" s="0" t="s">
-        <x:v>19</x:v>
+        <x:v>12</x:v>
       </x:c>
     </x:row>
     <x:row r="216" spans="1:11">
@@ -9028,7 +9031,7 @@
         <x:v>0.93</x:v>
       </x:c>
       <x:c r="I216" s="0">
-        <x:v>45.36</x:v>
+        <x:v>43</x:v>
       </x:c>
       <x:c r="J216" s="0">
         <x:v>30.45</x:v>
@@ -9063,7 +9066,7 @@
         <x:v>1.98</x:v>
       </x:c>
       <x:c r="I217" s="0">
-        <x:v>17.55</x:v>
+        <x:v>17.33</x:v>
       </x:c>
       <x:c r="J217" s="0">
         <x:v>11.47</x:v>
@@ -9098,7 +9101,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="I218" s="0">
-        <x:v>1.99</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="J218" s="0">
         <x:v>0</x:v>
@@ -9130,7 +9133,7 @@
         <x:v>0.21</x:v>
       </x:c>
       <x:c r="I219" s="0">
-        <x:v>9.3</x:v>
+        <x:v>9.54</x:v>
       </x:c>
       <x:c r="J219" s="0">
         <x:v>7.82</x:v>
@@ -9165,7 +9168,7 @@
         <x:v>0.15</x:v>
       </x:c>
       <x:c r="I220" s="0">
-        <x:v>13.24</x:v>
+        <x:v>13.34</x:v>
       </x:c>
       <x:c r="J220" s="0">
         <x:v>18.44</x:v>
@@ -9200,7 +9203,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="I221" s="0">
-        <x:v>27.26</x:v>
+        <x:v>28.06</x:v>
       </x:c>
       <x:c r="J221" s="0">
         <x:v>0</x:v>
@@ -9232,7 +9235,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="I222" s="0">
-        <x:v>519.5</x:v>
+        <x:v>520</x:v>
       </x:c>
       <x:c r="J222" s="0">
         <x:v>0</x:v>
@@ -9264,7 +9267,7 @@
         <x:v>0.03</x:v>
       </x:c>
       <x:c r="I223" s="0">
-        <x:v>229.5</x:v>
+        <x:v>230.6</x:v>
       </x:c>
       <x:c r="J223" s="0">
         <x:v>154.36</x:v>
@@ -9299,7 +9302,7 @@
         <x:v>0.33</x:v>
       </x:c>
       <x:c r="I224" s="0">
-        <x:v>5.5</x:v>
+        <x:v>6.05</x:v>
       </x:c>
       <x:c r="J224" s="0">
         <x:v>14.81</x:v>
@@ -9334,7 +9337,7 @@
         <x:v>0.25</x:v>
       </x:c>
       <x:c r="I225" s="0">
-        <x:v>0.99</x:v>
+        <x:v>1.01</x:v>
       </x:c>
       <x:c r="J225" s="0">
         <x:v>13.82</x:v>
@@ -9369,7 +9372,7 @@
         <x:v>0.26</x:v>
       </x:c>
       <x:c r="I226" s="0">
-        <x:v>5.03</x:v>
+        <x:v>4.92</x:v>
       </x:c>
       <x:c r="J226" s="0">
         <x:v>7.15</x:v>
@@ -9404,7 +9407,7 @@
         <x:v>0.06</x:v>
       </x:c>
       <x:c r="I227" s="0">
-        <x:v>519.5</x:v>
+        <x:v>520</x:v>
       </x:c>
       <x:c r="J227" s="0">
         <x:v>242.84</x:v>
@@ -9439,7 +9442,7 @@
         <x:v>0.36</x:v>
       </x:c>
       <x:c r="I228" s="0">
-        <x:v>728.5</x:v>
+        <x:v>731</x:v>
       </x:c>
       <x:c r="J228" s="0">
         <x:v>226</x:v>
@@ -9474,7 +9477,7 @@
         <x:v>0.1</x:v>
       </x:c>
       <x:c r="I229" s="0">
-        <x:v>5.5</x:v>
+        <x:v>6.05</x:v>
       </x:c>
       <x:c r="J229" s="0">
         <x:v>14.11</x:v>
@@ -9509,7 +9512,7 @@
         <x:v>0.18</x:v>
       </x:c>
       <x:c r="I230" s="0">
-        <x:v>0.99</x:v>
+        <x:v>1.01</x:v>
       </x:c>
       <x:c r="J230" s="0">
         <x:v>14.58</x:v>
@@ -9544,7 +9547,7 @@
         <x:v>1.74</x:v>
       </x:c>
       <x:c r="I231" s="0">
-        <x:v>146.5</x:v>
+        <x:v>142.5</x:v>
       </x:c>
       <x:c r="J231" s="0">
         <x:v>138.38</x:v>
@@ -9579,7 +9582,7 @@
         <x:v>3.6</x:v>
       </x:c>
       <x:c r="I232" s="0">
-        <x:v>36.94</x:v>
+        <x:v>36.6</x:v>
       </x:c>
       <x:c r="J232" s="0">
         <x:v>43</x:v>
@@ -9614,7 +9617,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="I233" s="0">
-        <x:v>243.5</x:v>
+        <x:v>236.1</x:v>
       </x:c>
       <x:c r="J233" s="0">
         <x:v>0</x:v>
@@ -9646,7 +9649,7 @@
         <x:v>0.03</x:v>
       </x:c>
       <x:c r="I234" s="0">
-        <x:v>2.63</x:v>
+        <x:v>2.59</x:v>
       </x:c>
       <x:c r="J234" s="0">
         <x:v>11.89</x:v>
@@ -9681,7 +9684,7 @@
         <x:v>0.03</x:v>
       </x:c>
       <x:c r="I235" s="0">
-        <x:v>34.5</x:v>
+        <x:v>35.44</x:v>
       </x:c>
       <x:c r="J235" s="0">
         <x:v>94</x:v>
@@ -9698,7 +9701,7 @@
         <x:v>365</x:v>
       </x:c>
       <x:c r="C236" s="0">
-        <x:v>2565919</x:v>
+        <x:v>2791213</x:v>
       </x:c>
       <x:c r="D236" s="0">
         <x:v>4250000</x:v>
@@ -9707,30 +9710,30 @@
         <x:v>40000000</x:v>
       </x:c>
       <x:c r="F236" s="0">
-        <x:v>17221295</x:v>
+        <x:v>18742029</x:v>
       </x:c>
       <x:c r="G236" s="0">
         <x:v>5</x:v>
       </x:c>
       <x:c r="H236" s="0">
-        <x:v>3.02</x:v>
+        <x:v>3.28</x:v>
       </x:c>
       <x:c r="I236" s="0">
-        <x:v>6.75</x:v>
+        <x:v>6.89</x:v>
       </x:c>
       <x:c r="J236" s="0">
         <x:v>6.71</x:v>
       </x:c>
       <x:c r="K236" s="0" t="s">
-        <x:v>19</x:v>
+        <x:v>366</x:v>
       </x:c>
     </x:row>
     <x:row r="237" spans="1:11">
       <x:c r="A237" s="0" t="s">
-        <x:v>366</x:v>
+        <x:v>367</x:v>
       </x:c>
       <x:c r="B237" s="0" t="s">
-        <x:v>367</x:v>
+        <x:v>368</x:v>
       </x:c>
       <x:c r="C237" s="0">
         <x:v>15000000</x:v>
@@ -9751,21 +9754,21 @@
         <x:v>0.22</x:v>
       </x:c>
       <x:c r="I237" s="0">
-        <x:v>1.72</x:v>
+        <x:v>1.73</x:v>
       </x:c>
       <x:c r="J237" s="0">
         <x:v>1.6</x:v>
       </x:c>
       <x:c r="K237" s="0" t="s">
-        <x:v>368</x:v>
+        <x:v>369</x:v>
       </x:c>
     </x:row>
     <x:row r="238" spans="1:11">
       <x:c r="A238" s="0" t="s">
-        <x:v>369</x:v>
+        <x:v>370</x:v>
       </x:c>
       <x:c r="B238" s="0" t="s">
-        <x:v>370</x:v>
+        <x:v>371</x:v>
       </x:c>
       <x:c r="C238" s="0">
         <x:v>6397124</x:v>
@@ -9786,13 +9789,13 @@
         <x:v>0.21</x:v>
       </x:c>
       <x:c r="I238" s="0">
-        <x:v>3.05</x:v>
+        <x:v>3.08</x:v>
       </x:c>
       <x:c r="J238" s="0">
         <x:v>19.21</x:v>
       </x:c>
       <x:c r="K238" s="0" t="s">
-        <x:v>371</x:v>
+        <x:v>372</x:v>
       </x:c>
     </x:row>
     <x:row r="239" spans="1:11">
@@ -9800,7 +9803,7 @@
         <x:v>196</x:v>
       </x:c>
       <x:c r="B239" s="0" t="s">
-        <x:v>372</x:v>
+        <x:v>373</x:v>
       </x:c>
       <x:c r="C239" s="0">
         <x:v>17495257</x:v>
@@ -9821,21 +9824,21 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="I239" s="0">
-        <x:v>13.99</x:v>
+        <x:v>14.34</x:v>
       </x:c>
       <x:c r="J239" s="0">
         <x:v>23.4</x:v>
       </x:c>
       <x:c r="K239" s="0" t="s">
-        <x:v>373</x:v>
+        <x:v>374</x:v>
       </x:c>
     </x:row>
     <x:row r="240" spans="1:11">
       <x:c r="A240" s="0" t="s">
-        <x:v>374</x:v>
+        <x:v>375</x:v>
       </x:c>
       <x:c r="B240" s="0" t="s">
-        <x:v>375</x:v>
+        <x:v>376</x:v>
       </x:c>
       <x:c r="C240" s="0">
         <x:v>9350000</x:v>
@@ -9856,13 +9859,13 @@
         <x:v>1.1</x:v>
       </x:c>
       <x:c r="I240" s="0">
-        <x:v>2.1</x:v>
+        <x:v>2.25</x:v>
       </x:c>
       <x:c r="J240" s="0">
         <x:v>7.44</x:v>
       </x:c>
       <x:c r="K240" s="0" t="s">
-        <x:v>376</x:v>
+        <x:v>377</x:v>
       </x:c>
     </x:row>
     <x:row r="241" spans="1:11">
@@ -9870,7 +9873,7 @@
         <x:v>224</x:v>
       </x:c>
       <x:c r="B241" s="0" t="s">
-        <x:v>377</x:v>
+        <x:v>378</x:v>
       </x:c>
       <x:c r="C241" s="0">
         <x:v>1468255</x:v>
@@ -9891,13 +9894,13 @@
         <x:v>0.37</x:v>
       </x:c>
       <x:c r="I241" s="0">
-        <x:v>22.7</x:v>
+        <x:v>23.16</x:v>
       </x:c>
       <x:c r="J241" s="0">
         <x:v>51.7</x:v>
       </x:c>
       <x:c r="K241" s="0" t="s">
-        <x:v>378</x:v>
+        <x:v>379</x:v>
       </x:c>
     </x:row>
     <x:row r="242" spans="1:11">
@@ -9905,7 +9908,7 @@
         <x:v>89</x:v>
       </x:c>
       <x:c r="B242" s="0" t="s">
-        <x:v>379</x:v>
+        <x:v>380</x:v>
       </x:c>
       <x:c r="C242" s="0">
         <x:v>500000</x:v>
@@ -9940,7 +9943,7 @@
         <x:v>229</x:v>
       </x:c>
       <x:c r="B243" s="0" t="s">
-        <x:v>380</x:v>
+        <x:v>381</x:v>
       </x:c>
       <x:c r="C243" s="0">
         <x:v>725000</x:v>
@@ -9961,21 +9964,21 @@
         <x:v>0.2</x:v>
       </x:c>
       <x:c r="I243" s="0">
-        <x:v>29.3</x:v>
+        <x:v>29.62</x:v>
       </x:c>
       <x:c r="J243" s="0">
         <x:v>66.95</x:v>
       </x:c>
       <x:c r="K243" s="0" t="s">
-        <x:v>381</x:v>
+        <x:v>382</x:v>
       </x:c>
     </x:row>
     <x:row r="244" spans="1:11">
       <x:c r="A244" s="0" t="s">
-        <x:v>382</x:v>
+        <x:v>383</x:v>
       </x:c>
       <x:c r="B244" s="0" t="s">
-        <x:v>383</x:v>
+        <x:v>384</x:v>
       </x:c>
       <x:c r="C244" s="0">
         <x:v>841000</x:v>
@@ -9996,7 +9999,7 @@
         <x:v>0.61</x:v>
       </x:c>
       <x:c r="I244" s="0">
-        <x:v>35.3</x:v>
+        <x:v>35.48</x:v>
       </x:c>
       <x:c r="J244" s="0">
         <x:v>38.43</x:v>
@@ -10010,7 +10013,7 @@
         <x:v>254</x:v>
       </x:c>
       <x:c r="B245" s="0" t="s">
-        <x:v>384</x:v>
+        <x:v>385</x:v>
       </x:c>
       <x:c r="C245" s="0">
         <x:v>1060056</x:v>
@@ -10031,13 +10034,13 @@
         <x:v>0.44</x:v>
       </x:c>
       <x:c r="I245" s="0">
-        <x:v>207.4</x:v>
+        <x:v>213.8</x:v>
       </x:c>
       <x:c r="J245" s="0">
         <x:v>57.32</x:v>
       </x:c>
       <x:c r="K245" s="0" t="s">
-        <x:v>385</x:v>
+        <x:v>386</x:v>
       </x:c>
     </x:row>
     <x:row r="246" spans="1:11">
@@ -10045,7 +10048,7 @@
         <x:v>245</x:v>
       </x:c>
       <x:c r="B246" s="0" t="s">
-        <x:v>386</x:v>
+        <x:v>387</x:v>
       </x:c>
       <x:c r="C246" s="0">
         <x:v>132750000</x:v>
@@ -10066,7 +10069,7 @@
         <x:v>0.25</x:v>
       </x:c>
       <x:c r="I246" s="0">
-        <x:v>1.88</x:v>
+        <x:v>1.93</x:v>
       </x:c>
       <x:c r="J246" s="0">
         <x:v>4.26</x:v>
@@ -10077,10 +10080,10 @@
     </x:row>
     <x:row r="247" spans="1:11">
       <x:c r="A247" s="0" t="s">
-        <x:v>387</x:v>
+        <x:v>388</x:v>
       </x:c>
       <x:c r="B247" s="0" t="s">
-        <x:v>388</x:v>
+        <x:v>389</x:v>
       </x:c>
       <x:c r="C247" s="0">
         <x:v>373000</x:v>
@@ -10101,21 +10104,21 @@
         <x:v>0.02</x:v>
       </x:c>
       <x:c r="I247" s="0">
-        <x:v>4.85</x:v>
+        <x:v>5.03</x:v>
       </x:c>
       <x:c r="J247" s="0">
         <x:v>63.77</x:v>
       </x:c>
       <x:c r="K247" s="0" t="s">
-        <x:v>389</x:v>
+        <x:v>390</x:v>
       </x:c>
     </x:row>
     <x:row r="248" spans="1:11">
       <x:c r="A248" s="0" t="s">
-        <x:v>390</x:v>
+        <x:v>391</x:v>
       </x:c>
       <x:c r="B248" s="0" t="s">
-        <x:v>391</x:v>
+        <x:v>392</x:v>
       </x:c>
       <x:c r="C248" s="0">
         <x:v>10000000</x:v>
@@ -10136,13 +10139,13 @@
         <x:v>0.67</x:v>
       </x:c>
       <x:c r="I248" s="0">
-        <x:v>7.9</x:v>
+        <x:v>7.13</x:v>
       </x:c>
       <x:c r="J248" s="0">
         <x:v>13.33</x:v>
       </x:c>
       <x:c r="K248" s="0" t="s">
-        <x:v>392</x:v>
+        <x:v>393</x:v>
       </x:c>
     </x:row>
     <x:row r="249" spans="1:11">
@@ -10150,7 +10153,7 @@
         <x:v>116</x:v>
       </x:c>
       <x:c r="B249" s="0" t="s">
-        <x:v>393</x:v>
+        <x:v>394</x:v>
       </x:c>
       <x:c r="C249" s="0">
         <x:v>66142950</x:v>
@@ -10171,21 +10174,21 @@
         <x:v>2.71</x:v>
       </x:c>
       <x:c r="I249" s="0">
-        <x:v>4.03</x:v>
+        <x:v>3.66</x:v>
       </x:c>
       <x:c r="J249" s="0">
         <x:v>5.82</x:v>
       </x:c>
       <x:c r="K249" s="0" t="s">
-        <x:v>394</x:v>
+        <x:v>395</x:v>
       </x:c>
     </x:row>
     <x:row r="250" spans="1:11">
       <x:c r="A250" s="0" t="s">
-        <x:v>395</x:v>
+        <x:v>396</x:v>
       </x:c>
       <x:c r="B250" s="0" t="s">
-        <x:v>396</x:v>
+        <x:v>397</x:v>
       </x:c>
       <x:c r="C250" s="0">
         <x:v>3935266</x:v>
@@ -10206,7 +10209,7 @@
         <x:v>0.84</x:v>
       </x:c>
       <x:c r="I250" s="0">
-        <x:v>4.96</x:v>
+        <x:v>4.95</x:v>
       </x:c>
       <x:c r="J250" s="0">
         <x:v>12.25</x:v>

</xml_diff>